<commit_message>
sync(workvault): 2026-10-23 10:33 差分 2 件
</commit_message>
<xml_diff>
--- a/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/Pana-CIM管理手順書案_未承認.xlsx
+++ b/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/Pana-CIM管理手順書案_未承認.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nk365-my.sharepoint.com/personal/ss80751_ad_nkc_co_jp/Documents/ドキュメント/Work_Vault/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10360" documentId="13_ncr:1_{22133521-4050-492C-8145-0AE2EA6E1C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8209AE7-992F-4B35-B121-83C758419604}"/>
+  <xr:revisionPtr revIDLastSave="10362" documentId="13_ncr:1_{22133521-4050-492C-8145-0AE2EA6E1C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{410EB5A4-5E7A-4387-8134-E05B441F776E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" firstSheet="9" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="表紙" sheetId="18" r:id="rId1"/>
@@ -2083,79 +2083,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="3" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="26" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2197,6 +2124,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="3" applyFont="1" applyBorder="1"/>
@@ -2208,6 +2144,70 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="26" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -7318,102 +7318,102 @@
       </c>
       <c r="N1" s="26"/>
       <c r="O1" s="27"/>
-      <c r="P1" s="49"/>
-      <c r="Q1" s="50"/>
-      <c r="R1" s="50"/>
-      <c r="S1" s="50"/>
-      <c r="T1" s="50"/>
-      <c r="U1" s="50"/>
-      <c r="V1" s="51"/>
+      <c r="P1" s="91"/>
+      <c r="Q1" s="92"/>
+      <c r="R1" s="92"/>
+      <c r="S1" s="92"/>
+      <c r="T1" s="92"/>
+      <c r="U1" s="92"/>
+      <c r="V1" s="93"/>
       <c r="W1" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="X1" s="52" t="s">
+      <c r="X1" s="94" t="s">
         <v>336</v>
       </c>
-      <c r="Y1" s="53"/>
+      <c r="Y1" s="95"/>
     </row>
     <row r="2" spans="1:25" ht="58.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="30"/>
       <c r="B2" s="31"/>
-      <c r="D2" s="54" t="s">
+      <c r="D2" s="96" t="s">
         <v>337</v>
       </c>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
-      <c r="H2" s="55"/>
-      <c r="I2" s="55"/>
-      <c r="J2" s="55"/>
-      <c r="K2" s="55"/>
-      <c r="L2" s="55"/>
-      <c r="M2" s="55"/>
-      <c r="N2" s="55"/>
-      <c r="O2" s="55"/>
-      <c r="P2" s="55"/>
-      <c r="Q2" s="55"/>
-      <c r="R2" s="55"/>
-      <c r="S2" s="55"/>
-      <c r="T2" s="55"/>
-      <c r="U2" s="55"/>
-      <c r="V2" s="55"/>
-      <c r="W2" s="55"/>
+      <c r="E2" s="97"/>
+      <c r="F2" s="97"/>
+      <c r="G2" s="97"/>
+      <c r="H2" s="97"/>
+      <c r="I2" s="97"/>
+      <c r="J2" s="97"/>
+      <c r="K2" s="97"/>
+      <c r="L2" s="97"/>
+      <c r="M2" s="97"/>
+      <c r="N2" s="97"/>
+      <c r="O2" s="97"/>
+      <c r="P2" s="97"/>
+      <c r="Q2" s="97"/>
+      <c r="R2" s="97"/>
+      <c r="S2" s="97"/>
+      <c r="T2" s="97"/>
+      <c r="U2" s="97"/>
+      <c r="V2" s="97"/>
+      <c r="W2" s="97"/>
       <c r="X2" s="32"/>
       <c r="Y2" s="24"/>
     </row>
     <row r="3" spans="1:25" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="33"/>
       <c r="B3" s="34"/>
-      <c r="D3" s="56" t="s">
+      <c r="D3" s="98" t="s">
         <v>338</v>
       </c>
-      <c r="E3" s="56"/>
-      <c r="F3" s="56"/>
-      <c r="G3" s="56"/>
-      <c r="H3" s="56"/>
-      <c r="I3" s="56"/>
-      <c r="J3" s="56"/>
-      <c r="K3" s="56"/>
-      <c r="L3" s="56"/>
-      <c r="M3" s="56"/>
-      <c r="N3" s="56"/>
-      <c r="O3" s="56"/>
-      <c r="P3" s="56"/>
-      <c r="Q3" s="56"/>
-      <c r="R3" s="56"/>
-      <c r="S3" s="56"/>
-      <c r="T3" s="56"/>
-      <c r="U3" s="56"/>
-      <c r="V3" s="56"/>
-      <c r="W3" s="56"/>
+      <c r="E3" s="98"/>
+      <c r="F3" s="98"/>
+      <c r="G3" s="98"/>
+      <c r="H3" s="98"/>
+      <c r="I3" s="98"/>
+      <c r="J3" s="98"/>
+      <c r="K3" s="98"/>
+      <c r="L3" s="98"/>
+      <c r="M3" s="98"/>
+      <c r="N3" s="98"/>
+      <c r="O3" s="98"/>
+      <c r="P3" s="98"/>
+      <c r="Q3" s="98"/>
+      <c r="R3" s="98"/>
+      <c r="S3" s="98"/>
+      <c r="T3" s="98"/>
+      <c r="U3" s="98"/>
+      <c r="V3" s="98"/>
+      <c r="W3" s="98"/>
       <c r="X3" s="34"/>
       <c r="Y3" s="35"/>
     </row>
     <row r="4" spans="1:25" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="33"/>
       <c r="B4" s="34"/>
-      <c r="D4" s="56" t="s">
+      <c r="D4" s="98" t="s">
         <v>339</v>
       </c>
-      <c r="E4" s="56"/>
-      <c r="F4" s="56"/>
-      <c r="G4" s="56"/>
-      <c r="H4" s="56"/>
-      <c r="I4" s="56"/>
-      <c r="J4" s="56"/>
-      <c r="K4" s="56"/>
-      <c r="L4" s="56"/>
-      <c r="M4" s="56"/>
-      <c r="N4" s="56"/>
-      <c r="O4" s="56"/>
-      <c r="P4" s="56"/>
-      <c r="Q4" s="56"/>
-      <c r="R4" s="56"/>
-      <c r="S4" s="56"/>
-      <c r="T4" s="56"/>
-      <c r="U4" s="56"/>
-      <c r="V4" s="56"/>
-      <c r="W4" s="56"/>
+      <c r="E4" s="98"/>
+      <c r="F4" s="98"/>
+      <c r="G4" s="98"/>
+      <c r="H4" s="98"/>
+      <c r="I4" s="98"/>
+      <c r="J4" s="98"/>
+      <c r="K4" s="98"/>
+      <c r="L4" s="98"/>
+      <c r="M4" s="98"/>
+      <c r="N4" s="98"/>
+      <c r="O4" s="98"/>
+      <c r="P4" s="98"/>
+      <c r="Q4" s="98"/>
+      <c r="R4" s="98"/>
+      <c r="S4" s="98"/>
+      <c r="T4" s="98"/>
+      <c r="U4" s="98"/>
+      <c r="V4" s="98"/>
+      <c r="W4" s="98"/>
       <c r="X4" s="34"/>
       <c r="Y4" s="35"/>
     </row>
@@ -7457,21 +7457,21 @@
       <c r="K6" s="34"/>
       <c r="L6" s="37"/>
       <c r="M6" s="37"/>
-      <c r="O6" s="49" t="s">
+      <c r="O6" s="91" t="s">
         <v>340</v>
       </c>
-      <c r="P6" s="50"/>
-      <c r="Q6" s="51"/>
-      <c r="R6" s="49" t="s">
+      <c r="P6" s="92"/>
+      <c r="Q6" s="93"/>
+      <c r="R6" s="91" t="s">
         <v>341</v>
       </c>
-      <c r="S6" s="50"/>
-      <c r="T6" s="51"/>
-      <c r="U6" s="49" t="s">
+      <c r="S6" s="92"/>
+      <c r="T6" s="93"/>
+      <c r="U6" s="91" t="s">
         <v>342</v>
       </c>
-      <c r="V6" s="50"/>
-      <c r="W6" s="51"/>
+      <c r="V6" s="92"/>
+      <c r="W6" s="93"/>
       <c r="Y6" s="35"/>
     </row>
     <row r="7" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7488,15 +7488,15 @@
       <c r="K7" s="34"/>
       <c r="L7" s="37"/>
       <c r="M7" s="37"/>
-      <c r="O7" s="63"/>
-      <c r="P7" s="64"/>
-      <c r="Q7" s="65"/>
-      <c r="R7" s="63"/>
-      <c r="S7" s="64"/>
-      <c r="T7" s="65"/>
-      <c r="U7" s="63"/>
-      <c r="V7" s="64"/>
-      <c r="W7" s="65"/>
+      <c r="O7" s="82"/>
+      <c r="P7" s="83"/>
+      <c r="Q7" s="84"/>
+      <c r="R7" s="82"/>
+      <c r="S7" s="83"/>
+      <c r="T7" s="84"/>
+      <c r="U7" s="82"/>
+      <c r="V7" s="83"/>
+      <c r="W7" s="84"/>
       <c r="Y7" s="35"/>
     </row>
     <row r="8" spans="1:25" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -7513,15 +7513,15 @@
       <c r="K8" s="34"/>
       <c r="L8" s="37"/>
       <c r="M8" s="37"/>
-      <c r="O8" s="66"/>
-      <c r="P8" s="67"/>
-      <c r="Q8" s="68"/>
-      <c r="R8" s="66"/>
-      <c r="S8" s="67"/>
-      <c r="T8" s="68"/>
-      <c r="U8" s="66"/>
-      <c r="V8" s="67"/>
-      <c r="W8" s="68"/>
+      <c r="O8" s="85"/>
+      <c r="P8" s="86"/>
+      <c r="Q8" s="87"/>
+      <c r="R8" s="85"/>
+      <c r="S8" s="86"/>
+      <c r="T8" s="87"/>
+      <c r="U8" s="85"/>
+      <c r="V8" s="86"/>
+      <c r="W8" s="87"/>
       <c r="Y8" s="35"/>
     </row>
     <row r="9" spans="1:25" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -7565,18 +7565,18 @@
       <c r="L10" s="37"/>
       <c r="M10" s="37"/>
       <c r="N10" s="37"/>
-      <c r="P10" s="69" t="s">
+      <c r="P10" s="88" t="s">
         <v>343</v>
       </c>
-      <c r="Q10" s="69"/>
-      <c r="R10" s="69"/>
-      <c r="S10" s="70" t="s">
+      <c r="Q10" s="88"/>
+      <c r="R10" s="88"/>
+      <c r="S10" s="89" t="s">
         <v>344</v>
       </c>
-      <c r="T10" s="70"/>
-      <c r="U10" s="70"/>
-      <c r="V10" s="70"/>
-      <c r="W10" s="70"/>
+      <c r="T10" s="89"/>
+      <c r="U10" s="89"/>
+      <c r="V10" s="89"/>
+      <c r="W10" s="89"/>
       <c r="Y10" s="35"/>
     </row>
     <row r="11" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -7594,27 +7594,27 @@
       <c r="L11" s="37"/>
       <c r="M11" s="37"/>
       <c r="N11" s="37"/>
-      <c r="P11" s="57" t="s">
+      <c r="P11" s="80" t="s">
         <v>345</v>
       </c>
-      <c r="Q11" s="57"/>
-      <c r="R11" s="57"/>
-      <c r="S11" s="71" t="s">
+      <c r="Q11" s="80"/>
+      <c r="R11" s="80"/>
+      <c r="S11" s="90" t="s">
         <v>344</v>
       </c>
-      <c r="T11" s="71"/>
-      <c r="U11" s="71"/>
-      <c r="V11" s="71"/>
-      <c r="W11" s="71"/>
+      <c r="T11" s="90"/>
+      <c r="U11" s="90"/>
+      <c r="V11" s="90"/>
+      <c r="W11" s="90"/>
       <c r="Y11" s="35"/>
     </row>
     <row r="12" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="38"/>
-      <c r="P12" s="57" t="s">
+      <c r="P12" s="80" t="s">
         <v>346</v>
       </c>
-      <c r="Q12" s="57"/>
-      <c r="R12" s="57"/>
+      <c r="Q12" s="80"/>
+      <c r="R12" s="80"/>
       <c r="S12" s="39"/>
       <c r="T12" s="39"/>
       <c r="U12" s="40" t="s">
@@ -7636,642 +7636,642 @@
         <v>349</v>
       </c>
       <c r="B14" s="45"/>
-      <c r="C14" s="58"/>
-      <c r="D14" s="57"/>
-      <c r="E14" s="57"/>
-      <c r="F14" s="59"/>
-      <c r="G14" s="58"/>
-      <c r="H14" s="57"/>
-      <c r="I14" s="57"/>
-      <c r="J14" s="59"/>
-      <c r="K14" s="60"/>
-      <c r="L14" s="61"/>
-      <c r="M14" s="61"/>
-      <c r="N14" s="61"/>
-      <c r="O14" s="61"/>
-      <c r="P14" s="61"/>
-      <c r="Q14" s="62"/>
-      <c r="R14" s="58"/>
-      <c r="S14" s="59"/>
-      <c r="T14" s="58"/>
-      <c r="U14" s="57"/>
-      <c r="V14" s="57"/>
-      <c r="W14" s="59"/>
-      <c r="X14" s="58"/>
-      <c r="Y14" s="59"/>
+      <c r="C14" s="78"/>
+      <c r="D14" s="80"/>
+      <c r="E14" s="80"/>
+      <c r="F14" s="79"/>
+      <c r="G14" s="78"/>
+      <c r="H14" s="80"/>
+      <c r="I14" s="80"/>
+      <c r="J14" s="79"/>
+      <c r="K14" s="81"/>
+      <c r="L14" s="76"/>
+      <c r="M14" s="76"/>
+      <c r="N14" s="76"/>
+      <c r="O14" s="76"/>
+      <c r="P14" s="76"/>
+      <c r="Q14" s="77"/>
+      <c r="R14" s="78"/>
+      <c r="S14" s="79"/>
+      <c r="T14" s="78"/>
+      <c r="U14" s="80"/>
+      <c r="V14" s="80"/>
+      <c r="W14" s="79"/>
+      <c r="X14" s="78"/>
+      <c r="Y14" s="79"/>
     </row>
     <row r="15" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B15" s="45"/>
-      <c r="C15" s="58"/>
-      <c r="D15" s="57"/>
-      <c r="E15" s="57"/>
-      <c r="F15" s="59"/>
-      <c r="G15" s="58"/>
-      <c r="H15" s="57"/>
-      <c r="I15" s="57"/>
-      <c r="J15" s="59"/>
-      <c r="K15" s="60"/>
-      <c r="L15" s="61"/>
-      <c r="M15" s="61"/>
-      <c r="N15" s="61"/>
-      <c r="O15" s="61"/>
-      <c r="P15" s="61"/>
-      <c r="Q15" s="62"/>
-      <c r="R15" s="58"/>
-      <c r="S15" s="59"/>
-      <c r="T15" s="58"/>
-      <c r="U15" s="57"/>
-      <c r="V15" s="57"/>
-      <c r="W15" s="59"/>
-      <c r="X15" s="58"/>
-      <c r="Y15" s="59"/>
+      <c r="C15" s="78"/>
+      <c r="D15" s="80"/>
+      <c r="E15" s="80"/>
+      <c r="F15" s="79"/>
+      <c r="G15" s="78"/>
+      <c r="H15" s="80"/>
+      <c r="I15" s="80"/>
+      <c r="J15" s="79"/>
+      <c r="K15" s="81"/>
+      <c r="L15" s="76"/>
+      <c r="M15" s="76"/>
+      <c r="N15" s="76"/>
+      <c r="O15" s="76"/>
+      <c r="P15" s="76"/>
+      <c r="Q15" s="77"/>
+      <c r="R15" s="78"/>
+      <c r="S15" s="79"/>
+      <c r="T15" s="78"/>
+      <c r="U15" s="80"/>
+      <c r="V15" s="80"/>
+      <c r="W15" s="79"/>
+      <c r="X15" s="78"/>
+      <c r="Y15" s="79"/>
     </row>
     <row r="16" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B16" s="45"/>
-      <c r="C16" s="58"/>
-      <c r="D16" s="57"/>
-      <c r="E16" s="57"/>
-      <c r="F16" s="59"/>
-      <c r="G16" s="58"/>
-      <c r="H16" s="57"/>
-      <c r="I16" s="57"/>
-      <c r="J16" s="59"/>
-      <c r="K16" s="60"/>
-      <c r="L16" s="61"/>
-      <c r="M16" s="61"/>
-      <c r="N16" s="61"/>
-      <c r="O16" s="61"/>
-      <c r="P16" s="61"/>
-      <c r="Q16" s="62"/>
-      <c r="R16" s="58"/>
-      <c r="S16" s="59"/>
-      <c r="T16" s="58"/>
-      <c r="U16" s="57"/>
-      <c r="V16" s="57"/>
-      <c r="W16" s="59"/>
-      <c r="X16" s="58"/>
-      <c r="Y16" s="59"/>
+      <c r="C16" s="78"/>
+      <c r="D16" s="80"/>
+      <c r="E16" s="80"/>
+      <c r="F16" s="79"/>
+      <c r="G16" s="78"/>
+      <c r="H16" s="80"/>
+      <c r="I16" s="80"/>
+      <c r="J16" s="79"/>
+      <c r="K16" s="81"/>
+      <c r="L16" s="76"/>
+      <c r="M16" s="76"/>
+      <c r="N16" s="76"/>
+      <c r="O16" s="76"/>
+      <c r="P16" s="76"/>
+      <c r="Q16" s="77"/>
+      <c r="R16" s="78"/>
+      <c r="S16" s="79"/>
+      <c r="T16" s="78"/>
+      <c r="U16" s="80"/>
+      <c r="V16" s="80"/>
+      <c r="W16" s="79"/>
+      <c r="X16" s="78"/>
+      <c r="Y16" s="79"/>
     </row>
     <row r="17" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B17" s="45"/>
-      <c r="C17" s="58"/>
-      <c r="D17" s="57"/>
-      <c r="E17" s="57"/>
-      <c r="F17" s="59"/>
-      <c r="G17" s="58"/>
-      <c r="H17" s="57"/>
-      <c r="I17" s="57"/>
-      <c r="J17" s="59"/>
-      <c r="K17" s="60"/>
-      <c r="L17" s="61"/>
-      <c r="M17" s="61"/>
-      <c r="N17" s="61"/>
-      <c r="O17" s="61"/>
-      <c r="P17" s="61"/>
-      <c r="Q17" s="62"/>
-      <c r="R17" s="58"/>
-      <c r="S17" s="59"/>
-      <c r="T17" s="58"/>
-      <c r="U17" s="57"/>
-      <c r="V17" s="57"/>
-      <c r="W17" s="59"/>
-      <c r="X17" s="58"/>
-      <c r="Y17" s="59"/>
+      <c r="C17" s="78"/>
+      <c r="D17" s="80"/>
+      <c r="E17" s="80"/>
+      <c r="F17" s="79"/>
+      <c r="G17" s="78"/>
+      <c r="H17" s="80"/>
+      <c r="I17" s="80"/>
+      <c r="J17" s="79"/>
+      <c r="K17" s="81"/>
+      <c r="L17" s="76"/>
+      <c r="M17" s="76"/>
+      <c r="N17" s="76"/>
+      <c r="O17" s="76"/>
+      <c r="P17" s="76"/>
+      <c r="Q17" s="77"/>
+      <c r="R17" s="78"/>
+      <c r="S17" s="79"/>
+      <c r="T17" s="78"/>
+      <c r="U17" s="80"/>
+      <c r="V17" s="80"/>
+      <c r="W17" s="79"/>
+      <c r="X17" s="78"/>
+      <c r="Y17" s="79"/>
     </row>
     <row r="18" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B18" s="45"/>
-      <c r="C18" s="58"/>
-      <c r="D18" s="57"/>
-      <c r="E18" s="57"/>
-      <c r="F18" s="59"/>
-      <c r="G18" s="58"/>
-      <c r="H18" s="57"/>
-      <c r="I18" s="57"/>
-      <c r="J18" s="59"/>
-      <c r="K18" s="60"/>
-      <c r="L18" s="61"/>
-      <c r="M18" s="61"/>
-      <c r="N18" s="61"/>
-      <c r="O18" s="61"/>
-      <c r="P18" s="61"/>
-      <c r="Q18" s="62"/>
-      <c r="R18" s="58"/>
-      <c r="S18" s="59"/>
-      <c r="T18" s="58"/>
-      <c r="U18" s="57"/>
-      <c r="V18" s="57"/>
-      <c r="W18" s="59"/>
-      <c r="X18" s="58"/>
-      <c r="Y18" s="59"/>
+      <c r="C18" s="78"/>
+      <c r="D18" s="80"/>
+      <c r="E18" s="80"/>
+      <c r="F18" s="79"/>
+      <c r="G18" s="78"/>
+      <c r="H18" s="80"/>
+      <c r="I18" s="80"/>
+      <c r="J18" s="79"/>
+      <c r="K18" s="81"/>
+      <c r="L18" s="76"/>
+      <c r="M18" s="76"/>
+      <c r="N18" s="76"/>
+      <c r="O18" s="76"/>
+      <c r="P18" s="76"/>
+      <c r="Q18" s="77"/>
+      <c r="R18" s="78"/>
+      <c r="S18" s="79"/>
+      <c r="T18" s="78"/>
+      <c r="U18" s="80"/>
+      <c r="V18" s="80"/>
+      <c r="W18" s="79"/>
+      <c r="X18" s="78"/>
+      <c r="Y18" s="79"/>
     </row>
     <row r="19" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B19" s="45"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="57"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="59"/>
-      <c r="G19" s="58"/>
-      <c r="H19" s="57"/>
-      <c r="I19" s="57"/>
-      <c r="J19" s="59"/>
-      <c r="K19" s="60"/>
-      <c r="L19" s="61"/>
-      <c r="M19" s="61"/>
-      <c r="N19" s="61"/>
-      <c r="O19" s="61"/>
-      <c r="P19" s="61"/>
-      <c r="Q19" s="62"/>
-      <c r="R19" s="58"/>
-      <c r="S19" s="59"/>
-      <c r="T19" s="58"/>
-      <c r="U19" s="57"/>
-      <c r="V19" s="57"/>
-      <c r="W19" s="59"/>
-      <c r="X19" s="58"/>
-      <c r="Y19" s="59"/>
+      <c r="C19" s="78"/>
+      <c r="D19" s="80"/>
+      <c r="E19" s="80"/>
+      <c r="F19" s="79"/>
+      <c r="G19" s="78"/>
+      <c r="H19" s="80"/>
+      <c r="I19" s="80"/>
+      <c r="J19" s="79"/>
+      <c r="K19" s="81"/>
+      <c r="L19" s="76"/>
+      <c r="M19" s="76"/>
+      <c r="N19" s="76"/>
+      <c r="O19" s="76"/>
+      <c r="P19" s="76"/>
+      <c r="Q19" s="77"/>
+      <c r="R19" s="78"/>
+      <c r="S19" s="79"/>
+      <c r="T19" s="78"/>
+      <c r="U19" s="80"/>
+      <c r="V19" s="80"/>
+      <c r="W19" s="79"/>
+      <c r="X19" s="78"/>
+      <c r="Y19" s="79"/>
     </row>
     <row r="20" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B20" s="45"/>
-      <c r="C20" s="58"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="59"/>
-      <c r="G20" s="58"/>
-      <c r="H20" s="57"/>
-      <c r="I20" s="57"/>
-      <c r="J20" s="59"/>
-      <c r="K20" s="60"/>
-      <c r="L20" s="61"/>
-      <c r="M20" s="61"/>
-      <c r="N20" s="61"/>
-      <c r="O20" s="61"/>
-      <c r="P20" s="61"/>
-      <c r="Q20" s="62"/>
-      <c r="R20" s="58"/>
-      <c r="S20" s="59"/>
-      <c r="T20" s="58"/>
-      <c r="U20" s="57"/>
-      <c r="V20" s="57"/>
-      <c r="W20" s="59"/>
-      <c r="X20" s="58"/>
-      <c r="Y20" s="59"/>
+      <c r="C20" s="78"/>
+      <c r="D20" s="80"/>
+      <c r="E20" s="80"/>
+      <c r="F20" s="79"/>
+      <c r="G20" s="78"/>
+      <c r="H20" s="80"/>
+      <c r="I20" s="80"/>
+      <c r="J20" s="79"/>
+      <c r="K20" s="81"/>
+      <c r="L20" s="76"/>
+      <c r="M20" s="76"/>
+      <c r="N20" s="76"/>
+      <c r="O20" s="76"/>
+      <c r="P20" s="76"/>
+      <c r="Q20" s="77"/>
+      <c r="R20" s="78"/>
+      <c r="S20" s="79"/>
+      <c r="T20" s="78"/>
+      <c r="U20" s="80"/>
+      <c r="V20" s="80"/>
+      <c r="W20" s="79"/>
+      <c r="X20" s="78"/>
+      <c r="Y20" s="79"/>
     </row>
     <row r="21" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B21" s="45"/>
-      <c r="C21" s="58"/>
-      <c r="D21" s="57"/>
-      <c r="E21" s="57"/>
-      <c r="F21" s="59"/>
-      <c r="G21" s="58"/>
-      <c r="H21" s="57"/>
-      <c r="I21" s="57"/>
-      <c r="J21" s="59"/>
-      <c r="K21" s="60"/>
-      <c r="L21" s="61"/>
-      <c r="M21" s="61"/>
-      <c r="N21" s="61"/>
-      <c r="O21" s="61"/>
-      <c r="P21" s="61"/>
-      <c r="Q21" s="62"/>
-      <c r="R21" s="58"/>
-      <c r="S21" s="59"/>
-      <c r="T21" s="58"/>
-      <c r="U21" s="57"/>
-      <c r="V21" s="57"/>
-      <c r="W21" s="59"/>
-      <c r="X21" s="58"/>
-      <c r="Y21" s="59"/>
+      <c r="C21" s="78"/>
+      <c r="D21" s="80"/>
+      <c r="E21" s="80"/>
+      <c r="F21" s="79"/>
+      <c r="G21" s="78"/>
+      <c r="H21" s="80"/>
+      <c r="I21" s="80"/>
+      <c r="J21" s="79"/>
+      <c r="K21" s="81"/>
+      <c r="L21" s="76"/>
+      <c r="M21" s="76"/>
+      <c r="N21" s="76"/>
+      <c r="O21" s="76"/>
+      <c r="P21" s="76"/>
+      <c r="Q21" s="77"/>
+      <c r="R21" s="78"/>
+      <c r="S21" s="79"/>
+      <c r="T21" s="78"/>
+      <c r="U21" s="80"/>
+      <c r="V21" s="80"/>
+      <c r="W21" s="79"/>
+      <c r="X21" s="78"/>
+      <c r="Y21" s="79"/>
     </row>
     <row r="22" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B22" s="45"/>
-      <c r="C22" s="58"/>
-      <c r="D22" s="57"/>
-      <c r="E22" s="57"/>
-      <c r="F22" s="59"/>
-      <c r="G22" s="58"/>
-      <c r="H22" s="57"/>
-      <c r="I22" s="57"/>
-      <c r="J22" s="59"/>
-      <c r="K22" s="60"/>
-      <c r="L22" s="61"/>
-      <c r="M22" s="61"/>
-      <c r="N22" s="61"/>
-      <c r="O22" s="61"/>
-      <c r="P22" s="61"/>
-      <c r="Q22" s="62"/>
-      <c r="R22" s="58"/>
-      <c r="S22" s="59"/>
-      <c r="T22" s="58"/>
-      <c r="U22" s="57"/>
-      <c r="V22" s="57"/>
-      <c r="W22" s="59"/>
-      <c r="X22" s="58"/>
-      <c r="Y22" s="59"/>
+      <c r="C22" s="78"/>
+      <c r="D22" s="80"/>
+      <c r="E22" s="80"/>
+      <c r="F22" s="79"/>
+      <c r="G22" s="78"/>
+      <c r="H22" s="80"/>
+      <c r="I22" s="80"/>
+      <c r="J22" s="79"/>
+      <c r="K22" s="81"/>
+      <c r="L22" s="76"/>
+      <c r="M22" s="76"/>
+      <c r="N22" s="76"/>
+      <c r="O22" s="76"/>
+      <c r="P22" s="76"/>
+      <c r="Q22" s="77"/>
+      <c r="R22" s="78"/>
+      <c r="S22" s="79"/>
+      <c r="T22" s="78"/>
+      <c r="U22" s="80"/>
+      <c r="V22" s="80"/>
+      <c r="W22" s="79"/>
+      <c r="X22" s="78"/>
+      <c r="Y22" s="79"/>
     </row>
     <row r="23" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B23" s="45"/>
-      <c r="C23" s="58"/>
-      <c r="D23" s="57"/>
-      <c r="E23" s="57"/>
-      <c r="F23" s="59"/>
-      <c r="G23" s="58"/>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
-      <c r="J23" s="59"/>
-      <c r="K23" s="60"/>
-      <c r="L23" s="61"/>
-      <c r="M23" s="61"/>
-      <c r="N23" s="61"/>
-      <c r="O23" s="61"/>
-      <c r="P23" s="61"/>
-      <c r="Q23" s="62"/>
-      <c r="R23" s="58"/>
-      <c r="S23" s="59"/>
-      <c r="T23" s="58"/>
-      <c r="U23" s="57"/>
-      <c r="V23" s="57"/>
-      <c r="W23" s="59"/>
-      <c r="X23" s="58"/>
-      <c r="Y23" s="59"/>
+      <c r="C23" s="78"/>
+      <c r="D23" s="80"/>
+      <c r="E23" s="80"/>
+      <c r="F23" s="79"/>
+      <c r="G23" s="78"/>
+      <c r="H23" s="80"/>
+      <c r="I23" s="80"/>
+      <c r="J23" s="79"/>
+      <c r="K23" s="81"/>
+      <c r="L23" s="76"/>
+      <c r="M23" s="76"/>
+      <c r="N23" s="76"/>
+      <c r="O23" s="76"/>
+      <c r="P23" s="76"/>
+      <c r="Q23" s="77"/>
+      <c r="R23" s="78"/>
+      <c r="S23" s="79"/>
+      <c r="T23" s="78"/>
+      <c r="U23" s="80"/>
+      <c r="V23" s="80"/>
+      <c r="W23" s="79"/>
+      <c r="X23" s="78"/>
+      <c r="Y23" s="79"/>
     </row>
     <row r="24" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B24" s="45"/>
-      <c r="C24" s="58"/>
-      <c r="D24" s="57"/>
-      <c r="E24" s="57"/>
-      <c r="F24" s="59"/>
-      <c r="G24" s="58"/>
-      <c r="H24" s="57"/>
-      <c r="I24" s="57"/>
-      <c r="J24" s="59"/>
-      <c r="K24" s="60"/>
-      <c r="L24" s="61"/>
-      <c r="M24" s="61"/>
-      <c r="N24" s="61"/>
-      <c r="O24" s="61"/>
-      <c r="P24" s="61"/>
-      <c r="Q24" s="62"/>
-      <c r="R24" s="58"/>
-      <c r="S24" s="59"/>
-      <c r="T24" s="58"/>
-      <c r="U24" s="57"/>
-      <c r="V24" s="57"/>
-      <c r="W24" s="59"/>
-      <c r="X24" s="58"/>
-      <c r="Y24" s="59"/>
+      <c r="C24" s="78"/>
+      <c r="D24" s="80"/>
+      <c r="E24" s="80"/>
+      <c r="F24" s="79"/>
+      <c r="G24" s="78"/>
+      <c r="H24" s="80"/>
+      <c r="I24" s="80"/>
+      <c r="J24" s="79"/>
+      <c r="K24" s="81"/>
+      <c r="L24" s="76"/>
+      <c r="M24" s="76"/>
+      <c r="N24" s="76"/>
+      <c r="O24" s="76"/>
+      <c r="P24" s="76"/>
+      <c r="Q24" s="77"/>
+      <c r="R24" s="78"/>
+      <c r="S24" s="79"/>
+      <c r="T24" s="78"/>
+      <c r="U24" s="80"/>
+      <c r="V24" s="80"/>
+      <c r="W24" s="79"/>
+      <c r="X24" s="78"/>
+      <c r="Y24" s="79"/>
     </row>
     <row r="25" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B25" s="45"/>
-      <c r="C25" s="58"/>
-      <c r="D25" s="57"/>
-      <c r="E25" s="57"/>
-      <c r="F25" s="59"/>
-      <c r="G25" s="58"/>
-      <c r="H25" s="57"/>
-      <c r="I25" s="57"/>
-      <c r="J25" s="59"/>
-      <c r="K25" s="60"/>
-      <c r="L25" s="61"/>
-      <c r="M25" s="61"/>
-      <c r="N25" s="61"/>
-      <c r="O25" s="61"/>
-      <c r="P25" s="61"/>
-      <c r="Q25" s="62"/>
-      <c r="R25" s="58"/>
-      <c r="S25" s="59"/>
-      <c r="T25" s="58"/>
-      <c r="U25" s="57"/>
-      <c r="V25" s="57"/>
-      <c r="W25" s="59"/>
-      <c r="X25" s="58"/>
-      <c r="Y25" s="59"/>
+      <c r="C25" s="78"/>
+      <c r="D25" s="80"/>
+      <c r="E25" s="80"/>
+      <c r="F25" s="79"/>
+      <c r="G25" s="78"/>
+      <c r="H25" s="80"/>
+      <c r="I25" s="80"/>
+      <c r="J25" s="79"/>
+      <c r="K25" s="81"/>
+      <c r="L25" s="76"/>
+      <c r="M25" s="76"/>
+      <c r="N25" s="76"/>
+      <c r="O25" s="76"/>
+      <c r="P25" s="76"/>
+      <c r="Q25" s="77"/>
+      <c r="R25" s="78"/>
+      <c r="S25" s="79"/>
+      <c r="T25" s="78"/>
+      <c r="U25" s="80"/>
+      <c r="V25" s="80"/>
+      <c r="W25" s="79"/>
+      <c r="X25" s="78"/>
+      <c r="Y25" s="79"/>
     </row>
     <row r="26" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B26" s="45"/>
-      <c r="C26" s="58"/>
-      <c r="D26" s="57"/>
-      <c r="E26" s="57"/>
-      <c r="F26" s="59"/>
-      <c r="G26" s="58"/>
-      <c r="H26" s="57"/>
-      <c r="I26" s="57"/>
-      <c r="J26" s="59"/>
-      <c r="K26" s="60"/>
-      <c r="L26" s="61"/>
-      <c r="M26" s="61"/>
-      <c r="N26" s="61"/>
-      <c r="O26" s="61"/>
-      <c r="P26" s="61"/>
-      <c r="Q26" s="62"/>
-      <c r="R26" s="58"/>
-      <c r="S26" s="59"/>
-      <c r="T26" s="58"/>
-      <c r="U26" s="57"/>
-      <c r="V26" s="57"/>
-      <c r="W26" s="59"/>
-      <c r="X26" s="58"/>
-      <c r="Y26" s="59"/>
+      <c r="C26" s="78"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="80"/>
+      <c r="F26" s="79"/>
+      <c r="G26" s="78"/>
+      <c r="H26" s="80"/>
+      <c r="I26" s="80"/>
+      <c r="J26" s="79"/>
+      <c r="K26" s="81"/>
+      <c r="L26" s="76"/>
+      <c r="M26" s="76"/>
+      <c r="N26" s="76"/>
+      <c r="O26" s="76"/>
+      <c r="P26" s="76"/>
+      <c r="Q26" s="77"/>
+      <c r="R26" s="78"/>
+      <c r="S26" s="79"/>
+      <c r="T26" s="78"/>
+      <c r="U26" s="80"/>
+      <c r="V26" s="80"/>
+      <c r="W26" s="79"/>
+      <c r="X26" s="78"/>
+      <c r="Y26" s="79"/>
     </row>
     <row r="27" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B27" s="45"/>
-      <c r="C27" s="58"/>
-      <c r="D27" s="57"/>
-      <c r="E27" s="57"/>
-      <c r="F27" s="59"/>
-      <c r="G27" s="58"/>
-      <c r="H27" s="57"/>
-      <c r="I27" s="57"/>
-      <c r="J27" s="59"/>
-      <c r="K27" s="60"/>
-      <c r="L27" s="61"/>
-      <c r="M27" s="61"/>
-      <c r="N27" s="61"/>
-      <c r="O27" s="61"/>
-      <c r="P27" s="61"/>
-      <c r="Q27" s="62"/>
-      <c r="R27" s="58"/>
-      <c r="S27" s="59"/>
-      <c r="T27" s="58"/>
-      <c r="U27" s="57"/>
-      <c r="V27" s="57"/>
-      <c r="W27" s="59"/>
-      <c r="X27" s="58"/>
-      <c r="Y27" s="59"/>
+      <c r="C27" s="78"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="80"/>
+      <c r="F27" s="79"/>
+      <c r="G27" s="78"/>
+      <c r="H27" s="80"/>
+      <c r="I27" s="80"/>
+      <c r="J27" s="79"/>
+      <c r="K27" s="81"/>
+      <c r="L27" s="76"/>
+      <c r="M27" s="76"/>
+      <c r="N27" s="76"/>
+      <c r="O27" s="76"/>
+      <c r="P27" s="76"/>
+      <c r="Q27" s="77"/>
+      <c r="R27" s="78"/>
+      <c r="S27" s="79"/>
+      <c r="T27" s="78"/>
+      <c r="U27" s="80"/>
+      <c r="V27" s="80"/>
+      <c r="W27" s="79"/>
+      <c r="X27" s="78"/>
+      <c r="Y27" s="79"/>
     </row>
     <row r="28" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B28" s="45"/>
-      <c r="C28" s="58"/>
-      <c r="D28" s="57"/>
-      <c r="E28" s="57"/>
-      <c r="F28" s="59"/>
-      <c r="G28" s="58"/>
-      <c r="H28" s="57"/>
-      <c r="I28" s="57"/>
-      <c r="J28" s="59"/>
-      <c r="K28" s="60"/>
-      <c r="L28" s="61"/>
-      <c r="M28" s="61"/>
-      <c r="N28" s="61"/>
-      <c r="O28" s="61"/>
-      <c r="P28" s="61"/>
-      <c r="Q28" s="62"/>
-      <c r="R28" s="58"/>
-      <c r="S28" s="59"/>
-      <c r="T28" s="58"/>
-      <c r="U28" s="57"/>
-      <c r="V28" s="57"/>
-      <c r="W28" s="59"/>
-      <c r="X28" s="58"/>
-      <c r="Y28" s="59"/>
+      <c r="C28" s="78"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="80"/>
+      <c r="F28" s="79"/>
+      <c r="G28" s="78"/>
+      <c r="H28" s="80"/>
+      <c r="I28" s="80"/>
+      <c r="J28" s="79"/>
+      <c r="K28" s="81"/>
+      <c r="L28" s="76"/>
+      <c r="M28" s="76"/>
+      <c r="N28" s="76"/>
+      <c r="O28" s="76"/>
+      <c r="P28" s="76"/>
+      <c r="Q28" s="77"/>
+      <c r="R28" s="78"/>
+      <c r="S28" s="79"/>
+      <c r="T28" s="78"/>
+      <c r="U28" s="80"/>
+      <c r="V28" s="80"/>
+      <c r="W28" s="79"/>
+      <c r="X28" s="78"/>
+      <c r="Y28" s="79"/>
     </row>
     <row r="29" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B29" s="45"/>
-      <c r="C29" s="58"/>
-      <c r="D29" s="57"/>
-      <c r="E29" s="57"/>
-      <c r="F29" s="59"/>
-      <c r="G29" s="58"/>
-      <c r="H29" s="57"/>
-      <c r="I29" s="57"/>
-      <c r="J29" s="59"/>
-      <c r="K29" s="60"/>
-      <c r="L29" s="61"/>
-      <c r="M29" s="61"/>
-      <c r="N29" s="61"/>
-      <c r="O29" s="61"/>
-      <c r="P29" s="61"/>
-      <c r="Q29" s="62"/>
-      <c r="R29" s="58"/>
-      <c r="S29" s="59"/>
-      <c r="T29" s="58"/>
-      <c r="U29" s="57"/>
-      <c r="V29" s="57"/>
-      <c r="W29" s="59"/>
-      <c r="X29" s="58"/>
-      <c r="Y29" s="59"/>
+      <c r="C29" s="78"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="80"/>
+      <c r="F29" s="79"/>
+      <c r="G29" s="78"/>
+      <c r="H29" s="80"/>
+      <c r="I29" s="80"/>
+      <c r="J29" s="79"/>
+      <c r="K29" s="81"/>
+      <c r="L29" s="76"/>
+      <c r="M29" s="76"/>
+      <c r="N29" s="76"/>
+      <c r="O29" s="76"/>
+      <c r="P29" s="76"/>
+      <c r="Q29" s="77"/>
+      <c r="R29" s="78"/>
+      <c r="S29" s="79"/>
+      <c r="T29" s="78"/>
+      <c r="U29" s="80"/>
+      <c r="V29" s="80"/>
+      <c r="W29" s="79"/>
+      <c r="X29" s="78"/>
+      <c r="Y29" s="79"/>
     </row>
     <row r="30" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="44" t="s">
         <v>349</v>
       </c>
       <c r="B30" s="45"/>
-      <c r="C30" s="58"/>
-      <c r="D30" s="57"/>
-      <c r="E30" s="57"/>
-      <c r="F30" s="59"/>
-      <c r="G30" s="58"/>
-      <c r="H30" s="57"/>
-      <c r="I30" s="57"/>
-      <c r="J30" s="59"/>
-      <c r="K30" s="60"/>
-      <c r="L30" s="61"/>
-      <c r="M30" s="61"/>
-      <c r="N30" s="61"/>
-      <c r="O30" s="61"/>
-      <c r="P30" s="61"/>
-      <c r="Q30" s="62"/>
-      <c r="R30" s="58"/>
-      <c r="S30" s="59"/>
-      <c r="T30" s="58"/>
-      <c r="U30" s="57"/>
-      <c r="V30" s="57"/>
-      <c r="W30" s="59"/>
-      <c r="X30" s="58"/>
-      <c r="Y30" s="59"/>
+      <c r="C30" s="78"/>
+      <c r="D30" s="80"/>
+      <c r="E30" s="80"/>
+      <c r="F30" s="79"/>
+      <c r="G30" s="78"/>
+      <c r="H30" s="80"/>
+      <c r="I30" s="80"/>
+      <c r="J30" s="79"/>
+      <c r="K30" s="81"/>
+      <c r="L30" s="76"/>
+      <c r="M30" s="76"/>
+      <c r="N30" s="76"/>
+      <c r="O30" s="76"/>
+      <c r="P30" s="76"/>
+      <c r="Q30" s="77"/>
+      <c r="R30" s="78"/>
+      <c r="S30" s="79"/>
+      <c r="T30" s="78"/>
+      <c r="U30" s="80"/>
+      <c r="V30" s="80"/>
+      <c r="W30" s="79"/>
+      <c r="X30" s="78"/>
+      <c r="Y30" s="79"/>
     </row>
     <row r="31" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="44"/>
       <c r="B31" s="45"/>
-      <c r="C31" s="72"/>
-      <c r="D31" s="73"/>
-      <c r="E31" s="73"/>
-      <c r="F31" s="74"/>
-      <c r="G31" s="72"/>
-      <c r="H31" s="73"/>
-      <c r="I31" s="73"/>
-      <c r="J31" s="74"/>
-      <c r="K31" s="60"/>
-      <c r="L31" s="61"/>
-      <c r="M31" s="61"/>
-      <c r="N31" s="61"/>
-      <c r="O31" s="61"/>
-      <c r="P31" s="61"/>
-      <c r="Q31" s="62"/>
-      <c r="R31" s="58"/>
-      <c r="S31" s="59"/>
-      <c r="T31" s="58"/>
-      <c r="U31" s="57"/>
-      <c r="V31" s="57"/>
-      <c r="W31" s="59"/>
-      <c r="X31" s="58"/>
-      <c r="Y31" s="59"/>
+      <c r="C31" s="66"/>
+      <c r="D31" s="67"/>
+      <c r="E31" s="67"/>
+      <c r="F31" s="68"/>
+      <c r="G31" s="66"/>
+      <c r="H31" s="67"/>
+      <c r="I31" s="67"/>
+      <c r="J31" s="68"/>
+      <c r="K31" s="81"/>
+      <c r="L31" s="76"/>
+      <c r="M31" s="76"/>
+      <c r="N31" s="76"/>
+      <c r="O31" s="76"/>
+      <c r="P31" s="76"/>
+      <c r="Q31" s="77"/>
+      <c r="R31" s="78"/>
+      <c r="S31" s="79"/>
+      <c r="T31" s="78"/>
+      <c r="U31" s="80"/>
+      <c r="V31" s="80"/>
+      <c r="W31" s="79"/>
+      <c r="X31" s="78"/>
+      <c r="Y31" s="79"/>
     </row>
     <row r="32" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="44"/>
       <c r="B32" s="45"/>
-      <c r="C32" s="72"/>
-      <c r="D32" s="73"/>
-      <c r="E32" s="73"/>
-      <c r="F32" s="74"/>
-      <c r="G32" s="72"/>
-      <c r="H32" s="73"/>
-      <c r="I32" s="73"/>
-      <c r="J32" s="74"/>
+      <c r="C32" s="66"/>
+      <c r="D32" s="67"/>
+      <c r="E32" s="67"/>
+      <c r="F32" s="68"/>
+      <c r="G32" s="66"/>
+      <c r="H32" s="67"/>
+      <c r="I32" s="67"/>
+      <c r="J32" s="68"/>
       <c r="K32" s="75"/>
-      <c r="L32" s="61"/>
-      <c r="M32" s="61"/>
-      <c r="N32" s="61"/>
-      <c r="O32" s="61"/>
-      <c r="P32" s="61"/>
-      <c r="Q32" s="62"/>
-      <c r="R32" s="58"/>
-      <c r="S32" s="59"/>
-      <c r="T32" s="58"/>
-      <c r="U32" s="57"/>
-      <c r="V32" s="57"/>
-      <c r="W32" s="59"/>
-      <c r="X32" s="58"/>
-      <c r="Y32" s="59"/>
+      <c r="L32" s="76"/>
+      <c r="M32" s="76"/>
+      <c r="N32" s="76"/>
+      <c r="O32" s="76"/>
+      <c r="P32" s="76"/>
+      <c r="Q32" s="77"/>
+      <c r="R32" s="78"/>
+      <c r="S32" s="79"/>
+      <c r="T32" s="78"/>
+      <c r="U32" s="80"/>
+      <c r="V32" s="80"/>
+      <c r="W32" s="79"/>
+      <c r="X32" s="78"/>
+      <c r="Y32" s="79"/>
     </row>
     <row r="33" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="46"/>
       <c r="B33" s="47"/>
-      <c r="C33" s="72"/>
-      <c r="D33" s="73"/>
-      <c r="E33" s="73"/>
-      <c r="F33" s="74"/>
-      <c r="G33" s="72"/>
-      <c r="H33" s="73"/>
-      <c r="I33" s="73"/>
-      <c r="J33" s="74"/>
-      <c r="K33" s="93"/>
-      <c r="L33" s="94"/>
-      <c r="M33" s="94"/>
-      <c r="N33" s="94"/>
-      <c r="O33" s="94"/>
-      <c r="P33" s="94"/>
-      <c r="Q33" s="95"/>
-      <c r="R33" s="96"/>
-      <c r="S33" s="97"/>
-      <c r="T33" s="96"/>
-      <c r="U33" s="98"/>
-      <c r="V33" s="98"/>
-      <c r="W33" s="97"/>
-      <c r="X33" s="96"/>
-      <c r="Y33" s="97"/>
+      <c r="C33" s="66"/>
+      <c r="D33" s="67"/>
+      <c r="E33" s="67"/>
+      <c r="F33" s="68"/>
+      <c r="G33" s="66"/>
+      <c r="H33" s="67"/>
+      <c r="I33" s="67"/>
+      <c r="J33" s="68"/>
+      <c r="K33" s="69"/>
+      <c r="L33" s="70"/>
+      <c r="M33" s="70"/>
+      <c r="N33" s="70"/>
+      <c r="O33" s="70"/>
+      <c r="P33" s="70"/>
+      <c r="Q33" s="71"/>
+      <c r="R33" s="72"/>
+      <c r="S33" s="73"/>
+      <c r="T33" s="72"/>
+      <c r="U33" s="74"/>
+      <c r="V33" s="74"/>
+      <c r="W33" s="73"/>
+      <c r="X33" s="72"/>
+      <c r="Y33" s="73"/>
     </row>
     <row r="34" spans="1:25" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="76" t="s">
+      <c r="A34" s="49" t="s">
         <v>350</v>
       </c>
-      <c r="B34" s="77"/>
-      <c r="C34" s="80" t="s">
+      <c r="B34" s="50"/>
+      <c r="C34" s="53" t="s">
         <v>351</v>
       </c>
-      <c r="D34" s="81"/>
-      <c r="E34" s="81"/>
-      <c r="F34" s="82"/>
-      <c r="G34" s="80" t="s">
+      <c r="D34" s="54"/>
+      <c r="E34" s="54"/>
+      <c r="F34" s="55"/>
+      <c r="G34" s="53" t="s">
         <v>352</v>
       </c>
-      <c r="H34" s="81"/>
-      <c r="I34" s="81"/>
-      <c r="J34" s="82"/>
-      <c r="K34" s="76" t="s">
+      <c r="H34" s="54"/>
+      <c r="I34" s="54"/>
+      <c r="J34" s="55"/>
+      <c r="K34" s="49" t="s">
         <v>353</v>
       </c>
-      <c r="L34" s="86"/>
-      <c r="M34" s="86"/>
-      <c r="N34" s="86"/>
-      <c r="O34" s="86"/>
-      <c r="P34" s="86"/>
-      <c r="Q34" s="87"/>
-      <c r="R34" s="76" t="s">
+      <c r="L34" s="59"/>
+      <c r="M34" s="59"/>
+      <c r="N34" s="59"/>
+      <c r="O34" s="59"/>
+      <c r="P34" s="59"/>
+      <c r="Q34" s="60"/>
+      <c r="R34" s="49" t="s">
         <v>354</v>
       </c>
-      <c r="S34" s="77"/>
-      <c r="T34" s="76" t="s">
+      <c r="S34" s="50"/>
+      <c r="T34" s="49" t="s">
         <v>355</v>
       </c>
-      <c r="U34" s="91"/>
-      <c r="V34" s="91"/>
-      <c r="W34" s="77"/>
-      <c r="X34" s="76" t="s">
+      <c r="U34" s="64"/>
+      <c r="V34" s="64"/>
+      <c r="W34" s="50"/>
+      <c r="X34" s="49" t="s">
         <v>356</v>
       </c>
-      <c r="Y34" s="77"/>
+      <c r="Y34" s="50"/>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A35" s="78"/>
-      <c r="B35" s="79"/>
-      <c r="C35" s="83"/>
-      <c r="D35" s="84"/>
-      <c r="E35" s="84"/>
-      <c r="F35" s="85"/>
-      <c r="G35" s="83"/>
-      <c r="H35" s="84"/>
-      <c r="I35" s="84"/>
-      <c r="J35" s="85"/>
-      <c r="K35" s="88"/>
-      <c r="L35" s="89"/>
-      <c r="M35" s="89"/>
-      <c r="N35" s="89"/>
-      <c r="O35" s="89"/>
-      <c r="P35" s="89"/>
-      <c r="Q35" s="90"/>
-      <c r="R35" s="78"/>
-      <c r="S35" s="79"/>
-      <c r="T35" s="78"/>
-      <c r="U35" s="92"/>
-      <c r="V35" s="92"/>
-      <c r="W35" s="79"/>
-      <c r="X35" s="78"/>
-      <c r="Y35" s="79"/>
+      <c r="A35" s="51"/>
+      <c r="B35" s="52"/>
+      <c r="C35" s="56"/>
+      <c r="D35" s="57"/>
+      <c r="E35" s="57"/>
+      <c r="F35" s="58"/>
+      <c r="G35" s="56"/>
+      <c r="H35" s="57"/>
+      <c r="I35" s="57"/>
+      <c r="J35" s="58"/>
+      <c r="K35" s="61"/>
+      <c r="L35" s="62"/>
+      <c r="M35" s="62"/>
+      <c r="N35" s="62"/>
+      <c r="O35" s="62"/>
+      <c r="P35" s="62"/>
+      <c r="Q35" s="63"/>
+      <c r="R35" s="51"/>
+      <c r="S35" s="52"/>
+      <c r="T35" s="51"/>
+      <c r="U35" s="65"/>
+      <c r="V35" s="65"/>
+      <c r="W35" s="52"/>
+      <c r="X35" s="51"/>
+      <c r="Y35" s="52"/>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A36" s="48" t="s">
@@ -8286,115 +8286,22 @@
     </row>
   </sheetData>
   <mergeCells count="143">
-    <mergeCell ref="X34:Y35"/>
-    <mergeCell ref="A34:B35"/>
-    <mergeCell ref="C34:F35"/>
-    <mergeCell ref="G34:J35"/>
-    <mergeCell ref="K34:Q35"/>
-    <mergeCell ref="R34:S35"/>
-    <mergeCell ref="T34:W35"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="G33:J33"/>
-    <mergeCell ref="K33:Q33"/>
-    <mergeCell ref="R33:S33"/>
-    <mergeCell ref="T33:W33"/>
-    <mergeCell ref="X33:Y33"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="G32:J32"/>
-    <mergeCell ref="K32:Q32"/>
-    <mergeCell ref="R32:S32"/>
-    <mergeCell ref="T32:W32"/>
-    <mergeCell ref="X32:Y32"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="K31:Q31"/>
-    <mergeCell ref="R31:S31"/>
-    <mergeCell ref="T31:W31"/>
-    <mergeCell ref="X31:Y31"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="K30:Q30"/>
-    <mergeCell ref="R30:S30"/>
-    <mergeCell ref="T30:W30"/>
-    <mergeCell ref="X30:Y30"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="K29:Q29"/>
-    <mergeCell ref="R29:S29"/>
-    <mergeCell ref="T29:W29"/>
-    <mergeCell ref="X29:Y29"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="K28:Q28"/>
-    <mergeCell ref="R28:S28"/>
-    <mergeCell ref="T28:W28"/>
-    <mergeCell ref="X28:Y28"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="G27:J27"/>
-    <mergeCell ref="K27:Q27"/>
-    <mergeCell ref="R27:S27"/>
-    <mergeCell ref="T27:W27"/>
-    <mergeCell ref="X27:Y27"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="K26:Q26"/>
-    <mergeCell ref="R26:S26"/>
-    <mergeCell ref="T26:W26"/>
-    <mergeCell ref="X26:Y26"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="K25:Q25"/>
-    <mergeCell ref="R25:S25"/>
-    <mergeCell ref="T25:W25"/>
-    <mergeCell ref="X25:Y25"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K24:Q24"/>
-    <mergeCell ref="R24:S24"/>
-    <mergeCell ref="T24:W24"/>
-    <mergeCell ref="X24:Y24"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="K23:Q23"/>
-    <mergeCell ref="R23:S23"/>
-    <mergeCell ref="T23:W23"/>
-    <mergeCell ref="X23:Y23"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="G22:J22"/>
-    <mergeCell ref="K22:Q22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="T22:W22"/>
-    <mergeCell ref="X22:Y22"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K21:Q21"/>
-    <mergeCell ref="R21:S21"/>
-    <mergeCell ref="T21:W21"/>
-    <mergeCell ref="X21:Y21"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="K20:Q20"/>
-    <mergeCell ref="R20:S20"/>
-    <mergeCell ref="T20:W20"/>
-    <mergeCell ref="X20:Y20"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="K19:Q19"/>
-    <mergeCell ref="R19:S19"/>
-    <mergeCell ref="T19:W19"/>
-    <mergeCell ref="X19:Y19"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="K18:Q18"/>
-    <mergeCell ref="R18:S18"/>
-    <mergeCell ref="T18:W18"/>
-    <mergeCell ref="X18:Y18"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="K17:Q17"/>
-    <mergeCell ref="R17:S17"/>
-    <mergeCell ref="T17:W17"/>
-    <mergeCell ref="X17:Y17"/>
+    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="O7:Q8"/>
+    <mergeCell ref="R7:T8"/>
+    <mergeCell ref="U7:W8"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="S10:W10"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="S11:W11"/>
+    <mergeCell ref="P1:V1"/>
+    <mergeCell ref="X1:Y1"/>
+    <mergeCell ref="D2:W2"/>
+    <mergeCell ref="D3:W3"/>
+    <mergeCell ref="D4:W4"/>
+    <mergeCell ref="O6:Q6"/>
+    <mergeCell ref="R6:T6"/>
+    <mergeCell ref="U6:W6"/>
     <mergeCell ref="C16:F16"/>
     <mergeCell ref="G16:J16"/>
     <mergeCell ref="K16:Q16"/>
@@ -8413,22 +8320,115 @@
     <mergeCell ref="K14:Q14"/>
     <mergeCell ref="R14:S14"/>
     <mergeCell ref="T14:W14"/>
-    <mergeCell ref="O7:Q8"/>
-    <mergeCell ref="R7:T8"/>
-    <mergeCell ref="U7:W8"/>
-    <mergeCell ref="P10:R10"/>
-    <mergeCell ref="S10:W10"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="S11:W11"/>
-    <mergeCell ref="P1:V1"/>
-    <mergeCell ref="X1:Y1"/>
-    <mergeCell ref="D2:W2"/>
-    <mergeCell ref="D3:W3"/>
-    <mergeCell ref="D4:W4"/>
-    <mergeCell ref="O6:Q6"/>
-    <mergeCell ref="R6:T6"/>
-    <mergeCell ref="U6:W6"/>
-    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="K18:Q18"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="T18:W18"/>
+    <mergeCell ref="X18:Y18"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="K17:Q17"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="T17:W17"/>
+    <mergeCell ref="X17:Y17"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="K20:Q20"/>
+    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="T20:W20"/>
+    <mergeCell ref="X20:Y20"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="K19:Q19"/>
+    <mergeCell ref="R19:S19"/>
+    <mergeCell ref="T19:W19"/>
+    <mergeCell ref="X19:Y19"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="G22:J22"/>
+    <mergeCell ref="K22:Q22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="T22:W22"/>
+    <mergeCell ref="X22:Y22"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K21:Q21"/>
+    <mergeCell ref="R21:S21"/>
+    <mergeCell ref="T21:W21"/>
+    <mergeCell ref="X21:Y21"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K24:Q24"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="T24:W24"/>
+    <mergeCell ref="X24:Y24"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="K23:Q23"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="T23:W23"/>
+    <mergeCell ref="X23:Y23"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="K26:Q26"/>
+    <mergeCell ref="R26:S26"/>
+    <mergeCell ref="T26:W26"/>
+    <mergeCell ref="X26:Y26"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="K25:Q25"/>
+    <mergeCell ref="R25:S25"/>
+    <mergeCell ref="T25:W25"/>
+    <mergeCell ref="X25:Y25"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="K28:Q28"/>
+    <mergeCell ref="R28:S28"/>
+    <mergeCell ref="T28:W28"/>
+    <mergeCell ref="X28:Y28"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="G27:J27"/>
+    <mergeCell ref="K27:Q27"/>
+    <mergeCell ref="R27:S27"/>
+    <mergeCell ref="T27:W27"/>
+    <mergeCell ref="X27:Y27"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="K30:Q30"/>
+    <mergeCell ref="R30:S30"/>
+    <mergeCell ref="T30:W30"/>
+    <mergeCell ref="X30:Y30"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="K29:Q29"/>
+    <mergeCell ref="R29:S29"/>
+    <mergeCell ref="T29:W29"/>
+    <mergeCell ref="X29:Y29"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="K32:Q32"/>
+    <mergeCell ref="R32:S32"/>
+    <mergeCell ref="T32:W32"/>
+    <mergeCell ref="X32:Y32"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="K31:Q31"/>
+    <mergeCell ref="R31:S31"/>
+    <mergeCell ref="T31:W31"/>
+    <mergeCell ref="X31:Y31"/>
+    <mergeCell ref="X34:Y35"/>
+    <mergeCell ref="A34:B35"/>
+    <mergeCell ref="C34:F35"/>
+    <mergeCell ref="G34:J35"/>
+    <mergeCell ref="K34:Q35"/>
+    <mergeCell ref="R34:S35"/>
+    <mergeCell ref="T34:W35"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="K33:Q33"/>
+    <mergeCell ref="R33:S33"/>
+    <mergeCell ref="T33:W33"/>
+    <mergeCell ref="X33:Y33"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.86614173228346458" right="0.51181102362204722" top="0.59055118110236227" bottom="0.19685039370078741" header="0.59055118110236227" footer="0.19685039370078741"/>

</xml_diff>

<commit_message>
sync(workvault): 2026-10-23 17:54 差分 5 件
</commit_message>
<xml_diff>
--- a/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/Pana-CIM管理手順書案_未承認.xlsx
+++ b/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/Pana-CIM管理手順書案_未承認.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nk365-my.sharepoint.com/personal/ss80751_ad_nkc_co_jp/Documents/ドキュメント/Work_Vault/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10560" documentId="13_ncr:1_{22133521-4050-492C-8145-0AE2EA6E1C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D54665DF-4627-41DD-A35E-F812ED673D25}"/>
+  <xr:revisionPtr revIDLastSave="10562" documentId="13_ncr:1_{22133521-4050-492C-8145-0AE2EA6E1C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7262B560-2756-4609-88E1-6181B043A5FC}"/>
   <bookViews>
     <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="10500" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2188,6 +2188,79 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="26" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2229,15 +2302,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="36" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="37" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="20" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="3" applyFont="1" applyBorder="1"/>
@@ -2248,70 +2312,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="21" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="26" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="32" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="11" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="24" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -9249,62 +9249,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>72543</xdr:colOff>
-      <xdr:row>106</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>35</xdr:col>
-      <xdr:colOff>83649</xdr:colOff>
-      <xdr:row>106</xdr:row>
-      <xdr:rowOff>15240</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="82" name="直線矢印コネクタ 81">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2FFF3187-F921-FB77-6305-90F78AAFA168}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3699663" y="17678400"/>
-          <a:ext cx="917886" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>29</xdr:col>
       <xdr:colOff>122848</xdr:colOff>
       <xdr:row>99</xdr:row>
@@ -9477,6 +9421,63 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>72543</xdr:colOff>
+      <xdr:row>106</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>35</xdr:col>
+      <xdr:colOff>83650</xdr:colOff>
+      <xdr:row>106</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="4" name="直線矢印コネクタ 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{74335EB5-48FF-944E-D451-9C056391D61A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="3699663" y="17678400"/>
+          <a:ext cx="917887" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:headEnd type="none"/>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -10433,102 +10434,102 @@
       </c>
       <c r="N1" s="26"/>
       <c r="O1" s="27"/>
-      <c r="P1" s="118"/>
-      <c r="Q1" s="119"/>
-      <c r="R1" s="119"/>
-      <c r="S1" s="119"/>
-      <c r="T1" s="119"/>
-      <c r="U1" s="119"/>
-      <c r="V1" s="120"/>
+      <c r="P1" s="90"/>
+      <c r="Q1" s="91"/>
+      <c r="R1" s="91"/>
+      <c r="S1" s="91"/>
+      <c r="T1" s="91"/>
+      <c r="U1" s="91"/>
+      <c r="V1" s="92"/>
       <c r="W1" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="X1" s="113" t="s">
+      <c r="X1" s="93" t="s">
         <v>298</v>
       </c>
-      <c r="Y1" s="114"/>
+      <c r="Y1" s="94"/>
     </row>
     <row r="2" spans="1:25" ht="58.5" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A2" s="30"/>
       <c r="B2" s="31"/>
-      <c r="D2" s="115" t="s">
+      <c r="D2" s="95" t="s">
         <v>299</v>
       </c>
-      <c r="E2" s="116"/>
-      <c r="F2" s="116"/>
-      <c r="G2" s="116"/>
-      <c r="H2" s="116"/>
-      <c r="I2" s="116"/>
-      <c r="J2" s="116"/>
-      <c r="K2" s="116"/>
-      <c r="L2" s="116"/>
-      <c r="M2" s="116"/>
-      <c r="N2" s="116"/>
-      <c r="O2" s="116"/>
-      <c r="P2" s="116"/>
-      <c r="Q2" s="116"/>
-      <c r="R2" s="116"/>
-      <c r="S2" s="116"/>
-      <c r="T2" s="116"/>
-      <c r="U2" s="116"/>
-      <c r="V2" s="116"/>
-      <c r="W2" s="116"/>
+      <c r="E2" s="96"/>
+      <c r="F2" s="96"/>
+      <c r="G2" s="96"/>
+      <c r="H2" s="96"/>
+      <c r="I2" s="96"/>
+      <c r="J2" s="96"/>
+      <c r="K2" s="96"/>
+      <c r="L2" s="96"/>
+      <c r="M2" s="96"/>
+      <c r="N2" s="96"/>
+      <c r="O2" s="96"/>
+      <c r="P2" s="96"/>
+      <c r="Q2" s="96"/>
+      <c r="R2" s="96"/>
+      <c r="S2" s="96"/>
+      <c r="T2" s="96"/>
+      <c r="U2" s="96"/>
+      <c r="V2" s="96"/>
+      <c r="W2" s="96"/>
       <c r="X2" s="32"/>
       <c r="Y2" s="24"/>
     </row>
     <row r="3" spans="1:25" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="33"/>
       <c r="B3" s="34"/>
-      <c r="D3" s="117" t="s">
+      <c r="D3" s="97" t="s">
         <v>300</v>
       </c>
-      <c r="E3" s="117"/>
-      <c r="F3" s="117"/>
-      <c r="G3" s="117"/>
-      <c r="H3" s="117"/>
-      <c r="I3" s="117"/>
-      <c r="J3" s="117"/>
-      <c r="K3" s="117"/>
-      <c r="L3" s="117"/>
-      <c r="M3" s="117"/>
-      <c r="N3" s="117"/>
-      <c r="O3" s="117"/>
-      <c r="P3" s="117"/>
-      <c r="Q3" s="117"/>
-      <c r="R3" s="117"/>
-      <c r="S3" s="117"/>
-      <c r="T3" s="117"/>
-      <c r="U3" s="117"/>
-      <c r="V3" s="117"/>
-      <c r="W3" s="117"/>
+      <c r="E3" s="97"/>
+      <c r="F3" s="97"/>
+      <c r="G3" s="97"/>
+      <c r="H3" s="97"/>
+      <c r="I3" s="97"/>
+      <c r="J3" s="97"/>
+      <c r="K3" s="97"/>
+      <c r="L3" s="97"/>
+      <c r="M3" s="97"/>
+      <c r="N3" s="97"/>
+      <c r="O3" s="97"/>
+      <c r="P3" s="97"/>
+      <c r="Q3" s="97"/>
+      <c r="R3" s="97"/>
+      <c r="S3" s="97"/>
+      <c r="T3" s="97"/>
+      <c r="U3" s="97"/>
+      <c r="V3" s="97"/>
+      <c r="W3" s="97"/>
       <c r="X3" s="34"/>
       <c r="Y3" s="35"/>
     </row>
     <row r="4" spans="1:25" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="33"/>
       <c r="B4" s="34"/>
-      <c r="D4" s="117" t="s">
+      <c r="D4" s="97" t="s">
         <v>301</v>
       </c>
-      <c r="E4" s="117"/>
-      <c r="F4" s="117"/>
-      <c r="G4" s="117"/>
-      <c r="H4" s="117"/>
-      <c r="I4" s="117"/>
-      <c r="J4" s="117"/>
-      <c r="K4" s="117"/>
-      <c r="L4" s="117"/>
-      <c r="M4" s="117"/>
-      <c r="N4" s="117"/>
-      <c r="O4" s="117"/>
-      <c r="P4" s="117"/>
-      <c r="Q4" s="117"/>
-      <c r="R4" s="117"/>
-      <c r="S4" s="117"/>
-      <c r="T4" s="117"/>
-      <c r="U4" s="117"/>
-      <c r="V4" s="117"/>
-      <c r="W4" s="117"/>
+      <c r="E4" s="97"/>
+      <c r="F4" s="97"/>
+      <c r="G4" s="97"/>
+      <c r="H4" s="97"/>
+      <c r="I4" s="97"/>
+      <c r="J4" s="97"/>
+      <c r="K4" s="97"/>
+      <c r="L4" s="97"/>
+      <c r="M4" s="97"/>
+      <c r="N4" s="97"/>
+      <c r="O4" s="97"/>
+      <c r="P4" s="97"/>
+      <c r="Q4" s="97"/>
+      <c r="R4" s="97"/>
+      <c r="S4" s="97"/>
+      <c r="T4" s="97"/>
+      <c r="U4" s="97"/>
+      <c r="V4" s="97"/>
+      <c r="W4" s="97"/>
       <c r="X4" s="34"/>
       <c r="Y4" s="35"/>
     </row>
@@ -10572,21 +10573,21 @@
       <c r="K6" s="34"/>
       <c r="L6" s="37"/>
       <c r="M6" s="37"/>
-      <c r="O6" s="118" t="s">
+      <c r="O6" s="90" t="s">
         <v>302</v>
       </c>
-      <c r="P6" s="119"/>
-      <c r="Q6" s="120"/>
-      <c r="R6" s="118" t="s">
+      <c r="P6" s="91"/>
+      <c r="Q6" s="92"/>
+      <c r="R6" s="90" t="s">
         <v>303</v>
       </c>
-      <c r="S6" s="119"/>
-      <c r="T6" s="120"/>
-      <c r="U6" s="118" t="s">
+      <c r="S6" s="91"/>
+      <c r="T6" s="92"/>
+      <c r="U6" s="90" t="s">
         <v>304</v>
       </c>
-      <c r="V6" s="119"/>
-      <c r="W6" s="120"/>
+      <c r="V6" s="91"/>
+      <c r="W6" s="92"/>
       <c r="Y6" s="35"/>
     </row>
     <row r="7" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -10603,15 +10604,15 @@
       <c r="K7" s="34"/>
       <c r="L7" s="37"/>
       <c r="M7" s="37"/>
-      <c r="O7" s="121"/>
-      <c r="P7" s="122"/>
-      <c r="Q7" s="123"/>
-      <c r="R7" s="121"/>
-      <c r="S7" s="122"/>
-      <c r="T7" s="123"/>
-      <c r="U7" s="121"/>
-      <c r="V7" s="122"/>
-      <c r="W7" s="123"/>
+      <c r="O7" s="81"/>
+      <c r="P7" s="82"/>
+      <c r="Q7" s="83"/>
+      <c r="R7" s="81"/>
+      <c r="S7" s="82"/>
+      <c r="T7" s="83"/>
+      <c r="U7" s="81"/>
+      <c r="V7" s="82"/>
+      <c r="W7" s="83"/>
       <c r="Y7" s="35"/>
     </row>
     <row r="8" spans="1:25" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
@@ -10628,15 +10629,15 @@
       <c r="K8" s="34"/>
       <c r="L8" s="37"/>
       <c r="M8" s="37"/>
-      <c r="O8" s="124"/>
-      <c r="P8" s="125"/>
-      <c r="Q8" s="126"/>
-      <c r="R8" s="124"/>
-      <c r="S8" s="125"/>
-      <c r="T8" s="126"/>
-      <c r="U8" s="124"/>
-      <c r="V8" s="125"/>
-      <c r="W8" s="126"/>
+      <c r="O8" s="84"/>
+      <c r="P8" s="85"/>
+      <c r="Q8" s="86"/>
+      <c r="R8" s="84"/>
+      <c r="S8" s="85"/>
+      <c r="T8" s="86"/>
+      <c r="U8" s="84"/>
+      <c r="V8" s="85"/>
+      <c r="W8" s="86"/>
       <c r="Y8" s="35"/>
     </row>
     <row r="9" spans="1:25" ht="6.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -10680,18 +10681,18 @@
       <c r="L10" s="37"/>
       <c r="M10" s="37"/>
       <c r="N10" s="37"/>
-      <c r="P10" s="127" t="s">
+      <c r="P10" s="87" t="s">
         <v>305</v>
       </c>
-      <c r="Q10" s="127"/>
-      <c r="R10" s="127"/>
-      <c r="S10" s="128" t="s">
+      <c r="Q10" s="87"/>
+      <c r="R10" s="87"/>
+      <c r="S10" s="88" t="s">
         <v>306</v>
       </c>
-      <c r="T10" s="128"/>
-      <c r="U10" s="128"/>
-      <c r="V10" s="128"/>
-      <c r="W10" s="128"/>
+      <c r="T10" s="88"/>
+      <c r="U10" s="88"/>
+      <c r="V10" s="88"/>
+      <c r="W10" s="88"/>
       <c r="Y10" s="35"/>
     </row>
     <row r="11" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
@@ -10709,27 +10710,27 @@
       <c r="L11" s="37"/>
       <c r="M11" s="37"/>
       <c r="N11" s="37"/>
-      <c r="P11" s="111" t="s">
+      <c r="P11" s="80" t="s">
         <v>307</v>
       </c>
-      <c r="Q11" s="111"/>
-      <c r="R11" s="111"/>
-      <c r="S11" s="129" t="s">
+      <c r="Q11" s="80"/>
+      <c r="R11" s="80"/>
+      <c r="S11" s="89" t="s">
         <v>306</v>
       </c>
-      <c r="T11" s="129"/>
-      <c r="U11" s="129"/>
-      <c r="V11" s="129"/>
-      <c r="W11" s="129"/>
+      <c r="T11" s="89"/>
+      <c r="U11" s="89"/>
+      <c r="V11" s="89"/>
+      <c r="W11" s="89"/>
       <c r="Y11" s="35"/>
     </row>
     <row r="12" spans="1:25" ht="32.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="38"/>
-      <c r="P12" s="111" t="s">
+      <c r="P12" s="80" t="s">
         <v>308</v>
       </c>
-      <c r="Q12" s="111"/>
-      <c r="R12" s="111"/>
+      <c r="Q12" s="80"/>
+      <c r="R12" s="80"/>
       <c r="S12" s="39"/>
       <c r="T12" s="39"/>
       <c r="U12" s="40" t="s">
@@ -10751,642 +10752,642 @@
         <v>311</v>
       </c>
       <c r="B14" s="45"/>
-      <c r="C14" s="109"/>
-      <c r="D14" s="111"/>
-      <c r="E14" s="111"/>
-      <c r="F14" s="110"/>
-      <c r="G14" s="109"/>
-      <c r="H14" s="111"/>
-      <c r="I14" s="111"/>
-      <c r="J14" s="110"/>
-      <c r="K14" s="112"/>
-      <c r="L14" s="107"/>
-      <c r="M14" s="107"/>
-      <c r="N14" s="107"/>
-      <c r="O14" s="107"/>
-      <c r="P14" s="107"/>
-      <c r="Q14" s="108"/>
-      <c r="R14" s="109"/>
-      <c r="S14" s="110"/>
-      <c r="T14" s="109"/>
-      <c r="U14" s="111"/>
-      <c r="V14" s="111"/>
-      <c r="W14" s="110"/>
-      <c r="X14" s="109"/>
-      <c r="Y14" s="110"/>
+      <c r="C14" s="98"/>
+      <c r="D14" s="80"/>
+      <c r="E14" s="80"/>
+      <c r="F14" s="99"/>
+      <c r="G14" s="98"/>
+      <c r="H14" s="80"/>
+      <c r="I14" s="80"/>
+      <c r="J14" s="99"/>
+      <c r="K14" s="100"/>
+      <c r="L14" s="101"/>
+      <c r="M14" s="101"/>
+      <c r="N14" s="101"/>
+      <c r="O14" s="101"/>
+      <c r="P14" s="101"/>
+      <c r="Q14" s="102"/>
+      <c r="R14" s="98"/>
+      <c r="S14" s="99"/>
+      <c r="T14" s="98"/>
+      <c r="U14" s="80"/>
+      <c r="V14" s="80"/>
+      <c r="W14" s="99"/>
+      <c r="X14" s="98"/>
+      <c r="Y14" s="99"/>
     </row>
     <row r="15" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B15" s="45"/>
-      <c r="C15" s="109"/>
-      <c r="D15" s="111"/>
-      <c r="E15" s="111"/>
-      <c r="F15" s="110"/>
-      <c r="G15" s="109"/>
-      <c r="H15" s="111"/>
-      <c r="I15" s="111"/>
-      <c r="J15" s="110"/>
-      <c r="K15" s="112"/>
-      <c r="L15" s="107"/>
-      <c r="M15" s="107"/>
-      <c r="N15" s="107"/>
-      <c r="O15" s="107"/>
-      <c r="P15" s="107"/>
-      <c r="Q15" s="108"/>
-      <c r="R15" s="109"/>
-      <c r="S15" s="110"/>
-      <c r="T15" s="109"/>
-      <c r="U15" s="111"/>
-      <c r="V15" s="111"/>
-      <c r="W15" s="110"/>
-      <c r="X15" s="109"/>
-      <c r="Y15" s="110"/>
+      <c r="C15" s="98"/>
+      <c r="D15" s="80"/>
+      <c r="E15" s="80"/>
+      <c r="F15" s="99"/>
+      <c r="G15" s="98"/>
+      <c r="H15" s="80"/>
+      <c r="I15" s="80"/>
+      <c r="J15" s="99"/>
+      <c r="K15" s="100"/>
+      <c r="L15" s="101"/>
+      <c r="M15" s="101"/>
+      <c r="N15" s="101"/>
+      <c r="O15" s="101"/>
+      <c r="P15" s="101"/>
+      <c r="Q15" s="102"/>
+      <c r="R15" s="98"/>
+      <c r="S15" s="99"/>
+      <c r="T15" s="98"/>
+      <c r="U15" s="80"/>
+      <c r="V15" s="80"/>
+      <c r="W15" s="99"/>
+      <c r="X15" s="98"/>
+      <c r="Y15" s="99"/>
     </row>
     <row r="16" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B16" s="45"/>
-      <c r="C16" s="109"/>
-      <c r="D16" s="111"/>
-      <c r="E16" s="111"/>
-      <c r="F16" s="110"/>
-      <c r="G16" s="109"/>
-      <c r="H16" s="111"/>
-      <c r="I16" s="111"/>
-      <c r="J16" s="110"/>
-      <c r="K16" s="112"/>
-      <c r="L16" s="107"/>
-      <c r="M16" s="107"/>
-      <c r="N16" s="107"/>
-      <c r="O16" s="107"/>
-      <c r="P16" s="107"/>
-      <c r="Q16" s="108"/>
-      <c r="R16" s="109"/>
-      <c r="S16" s="110"/>
-      <c r="T16" s="109"/>
-      <c r="U16" s="111"/>
-      <c r="V16" s="111"/>
-      <c r="W16" s="110"/>
-      <c r="X16" s="109"/>
-      <c r="Y16" s="110"/>
+      <c r="C16" s="98"/>
+      <c r="D16" s="80"/>
+      <c r="E16" s="80"/>
+      <c r="F16" s="99"/>
+      <c r="G16" s="98"/>
+      <c r="H16" s="80"/>
+      <c r="I16" s="80"/>
+      <c r="J16" s="99"/>
+      <c r="K16" s="100"/>
+      <c r="L16" s="101"/>
+      <c r="M16" s="101"/>
+      <c r="N16" s="101"/>
+      <c r="O16" s="101"/>
+      <c r="P16" s="101"/>
+      <c r="Q16" s="102"/>
+      <c r="R16" s="98"/>
+      <c r="S16" s="99"/>
+      <c r="T16" s="98"/>
+      <c r="U16" s="80"/>
+      <c r="V16" s="80"/>
+      <c r="W16" s="99"/>
+      <c r="X16" s="98"/>
+      <c r="Y16" s="99"/>
     </row>
     <row r="17" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B17" s="45"/>
-      <c r="C17" s="109"/>
-      <c r="D17" s="111"/>
-      <c r="E17" s="111"/>
-      <c r="F17" s="110"/>
-      <c r="G17" s="109"/>
-      <c r="H17" s="111"/>
-      <c r="I17" s="111"/>
-      <c r="J17" s="110"/>
-      <c r="K17" s="112"/>
-      <c r="L17" s="107"/>
-      <c r="M17" s="107"/>
-      <c r="N17" s="107"/>
-      <c r="O17" s="107"/>
-      <c r="P17" s="107"/>
-      <c r="Q17" s="108"/>
-      <c r="R17" s="109"/>
-      <c r="S17" s="110"/>
-      <c r="T17" s="109"/>
-      <c r="U17" s="111"/>
-      <c r="V17" s="111"/>
-      <c r="W17" s="110"/>
-      <c r="X17" s="109"/>
-      <c r="Y17" s="110"/>
+      <c r="C17" s="98"/>
+      <c r="D17" s="80"/>
+      <c r="E17" s="80"/>
+      <c r="F17" s="99"/>
+      <c r="G17" s="98"/>
+      <c r="H17" s="80"/>
+      <c r="I17" s="80"/>
+      <c r="J17" s="99"/>
+      <c r="K17" s="100"/>
+      <c r="L17" s="101"/>
+      <c r="M17" s="101"/>
+      <c r="N17" s="101"/>
+      <c r="O17" s="101"/>
+      <c r="P17" s="101"/>
+      <c r="Q17" s="102"/>
+      <c r="R17" s="98"/>
+      <c r="S17" s="99"/>
+      <c r="T17" s="98"/>
+      <c r="U17" s="80"/>
+      <c r="V17" s="80"/>
+      <c r="W17" s="99"/>
+      <c r="X17" s="98"/>
+      <c r="Y17" s="99"/>
     </row>
     <row r="18" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B18" s="45"/>
-      <c r="C18" s="109"/>
-      <c r="D18" s="111"/>
-      <c r="E18" s="111"/>
-      <c r="F18" s="110"/>
-      <c r="G18" s="109"/>
-      <c r="H18" s="111"/>
-      <c r="I18" s="111"/>
-      <c r="J18" s="110"/>
-      <c r="K18" s="112"/>
-      <c r="L18" s="107"/>
-      <c r="M18" s="107"/>
-      <c r="N18" s="107"/>
-      <c r="O18" s="107"/>
-      <c r="P18" s="107"/>
-      <c r="Q18" s="108"/>
-      <c r="R18" s="109"/>
-      <c r="S18" s="110"/>
-      <c r="T18" s="109"/>
-      <c r="U18" s="111"/>
-      <c r="V18" s="111"/>
-      <c r="W18" s="110"/>
-      <c r="X18" s="109"/>
-      <c r="Y18" s="110"/>
+      <c r="C18" s="98"/>
+      <c r="D18" s="80"/>
+      <c r="E18" s="80"/>
+      <c r="F18" s="99"/>
+      <c r="G18" s="98"/>
+      <c r="H18" s="80"/>
+      <c r="I18" s="80"/>
+      <c r="J18" s="99"/>
+      <c r="K18" s="100"/>
+      <c r="L18" s="101"/>
+      <c r="M18" s="101"/>
+      <c r="N18" s="101"/>
+      <c r="O18" s="101"/>
+      <c r="P18" s="101"/>
+      <c r="Q18" s="102"/>
+      <c r="R18" s="98"/>
+      <c r="S18" s="99"/>
+      <c r="T18" s="98"/>
+      <c r="U18" s="80"/>
+      <c r="V18" s="80"/>
+      <c r="W18" s="99"/>
+      <c r="X18" s="98"/>
+      <c r="Y18" s="99"/>
     </row>
     <row r="19" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B19" s="45"/>
-      <c r="C19" s="109"/>
-      <c r="D19" s="111"/>
-      <c r="E19" s="111"/>
-      <c r="F19" s="110"/>
-      <c r="G19" s="109"/>
-      <c r="H19" s="111"/>
-      <c r="I19" s="111"/>
-      <c r="J19" s="110"/>
-      <c r="K19" s="112"/>
-      <c r="L19" s="107"/>
-      <c r="M19" s="107"/>
-      <c r="N19" s="107"/>
-      <c r="O19" s="107"/>
-      <c r="P19" s="107"/>
-      <c r="Q19" s="108"/>
-      <c r="R19" s="109"/>
-      <c r="S19" s="110"/>
-      <c r="T19" s="109"/>
-      <c r="U19" s="111"/>
-      <c r="V19" s="111"/>
-      <c r="W19" s="110"/>
-      <c r="X19" s="109"/>
-      <c r="Y19" s="110"/>
+      <c r="C19" s="98"/>
+      <c r="D19" s="80"/>
+      <c r="E19" s="80"/>
+      <c r="F19" s="99"/>
+      <c r="G19" s="98"/>
+      <c r="H19" s="80"/>
+      <c r="I19" s="80"/>
+      <c r="J19" s="99"/>
+      <c r="K19" s="100"/>
+      <c r="L19" s="101"/>
+      <c r="M19" s="101"/>
+      <c r="N19" s="101"/>
+      <c r="O19" s="101"/>
+      <c r="P19" s="101"/>
+      <c r="Q19" s="102"/>
+      <c r="R19" s="98"/>
+      <c r="S19" s="99"/>
+      <c r="T19" s="98"/>
+      <c r="U19" s="80"/>
+      <c r="V19" s="80"/>
+      <c r="W19" s="99"/>
+      <c r="X19" s="98"/>
+      <c r="Y19" s="99"/>
     </row>
     <row r="20" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B20" s="45"/>
-      <c r="C20" s="109"/>
-      <c r="D20" s="111"/>
-      <c r="E20" s="111"/>
-      <c r="F20" s="110"/>
-      <c r="G20" s="109"/>
-      <c r="H20" s="111"/>
-      <c r="I20" s="111"/>
-      <c r="J20" s="110"/>
-      <c r="K20" s="112"/>
-      <c r="L20" s="107"/>
-      <c r="M20" s="107"/>
-      <c r="N20" s="107"/>
-      <c r="O20" s="107"/>
-      <c r="P20" s="107"/>
-      <c r="Q20" s="108"/>
-      <c r="R20" s="109"/>
-      <c r="S20" s="110"/>
-      <c r="T20" s="109"/>
-      <c r="U20" s="111"/>
-      <c r="V20" s="111"/>
-      <c r="W20" s="110"/>
-      <c r="X20" s="109"/>
-      <c r="Y20" s="110"/>
+      <c r="C20" s="98"/>
+      <c r="D20" s="80"/>
+      <c r="E20" s="80"/>
+      <c r="F20" s="99"/>
+      <c r="G20" s="98"/>
+      <c r="H20" s="80"/>
+      <c r="I20" s="80"/>
+      <c r="J20" s="99"/>
+      <c r="K20" s="100"/>
+      <c r="L20" s="101"/>
+      <c r="M20" s="101"/>
+      <c r="N20" s="101"/>
+      <c r="O20" s="101"/>
+      <c r="P20" s="101"/>
+      <c r="Q20" s="102"/>
+      <c r="R20" s="98"/>
+      <c r="S20" s="99"/>
+      <c r="T20" s="98"/>
+      <c r="U20" s="80"/>
+      <c r="V20" s="80"/>
+      <c r="W20" s="99"/>
+      <c r="X20" s="98"/>
+      <c r="Y20" s="99"/>
     </row>
     <row r="21" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B21" s="45"/>
-      <c r="C21" s="109"/>
-      <c r="D21" s="111"/>
-      <c r="E21" s="111"/>
-      <c r="F21" s="110"/>
-      <c r="G21" s="109"/>
-      <c r="H21" s="111"/>
-      <c r="I21" s="111"/>
-      <c r="J21" s="110"/>
-      <c r="K21" s="112"/>
-      <c r="L21" s="107"/>
-      <c r="M21" s="107"/>
-      <c r="N21" s="107"/>
-      <c r="O21" s="107"/>
-      <c r="P21" s="107"/>
-      <c r="Q21" s="108"/>
-      <c r="R21" s="109"/>
-      <c r="S21" s="110"/>
-      <c r="T21" s="109"/>
-      <c r="U21" s="111"/>
-      <c r="V21" s="111"/>
-      <c r="W21" s="110"/>
-      <c r="X21" s="109"/>
-      <c r="Y21" s="110"/>
+      <c r="C21" s="98"/>
+      <c r="D21" s="80"/>
+      <c r="E21" s="80"/>
+      <c r="F21" s="99"/>
+      <c r="G21" s="98"/>
+      <c r="H21" s="80"/>
+      <c r="I21" s="80"/>
+      <c r="J21" s="99"/>
+      <c r="K21" s="100"/>
+      <c r="L21" s="101"/>
+      <c r="M21" s="101"/>
+      <c r="N21" s="101"/>
+      <c r="O21" s="101"/>
+      <c r="P21" s="101"/>
+      <c r="Q21" s="102"/>
+      <c r="R21" s="98"/>
+      <c r="S21" s="99"/>
+      <c r="T21" s="98"/>
+      <c r="U21" s="80"/>
+      <c r="V21" s="80"/>
+      <c r="W21" s="99"/>
+      <c r="X21" s="98"/>
+      <c r="Y21" s="99"/>
     </row>
     <row r="22" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B22" s="45"/>
-      <c r="C22" s="109"/>
-      <c r="D22" s="111"/>
-      <c r="E22" s="111"/>
-      <c r="F22" s="110"/>
-      <c r="G22" s="109"/>
-      <c r="H22" s="111"/>
-      <c r="I22" s="111"/>
-      <c r="J22" s="110"/>
-      <c r="K22" s="112"/>
-      <c r="L22" s="107"/>
-      <c r="M22" s="107"/>
-      <c r="N22" s="107"/>
-      <c r="O22" s="107"/>
-      <c r="P22" s="107"/>
-      <c r="Q22" s="108"/>
-      <c r="R22" s="109"/>
-      <c r="S22" s="110"/>
-      <c r="T22" s="109"/>
-      <c r="U22" s="111"/>
-      <c r="V22" s="111"/>
-      <c r="W22" s="110"/>
-      <c r="X22" s="109"/>
-      <c r="Y22" s="110"/>
+      <c r="C22" s="98"/>
+      <c r="D22" s="80"/>
+      <c r="E22" s="80"/>
+      <c r="F22" s="99"/>
+      <c r="G22" s="98"/>
+      <c r="H22" s="80"/>
+      <c r="I22" s="80"/>
+      <c r="J22" s="99"/>
+      <c r="K22" s="100"/>
+      <c r="L22" s="101"/>
+      <c r="M22" s="101"/>
+      <c r="N22" s="101"/>
+      <c r="O22" s="101"/>
+      <c r="P22" s="101"/>
+      <c r="Q22" s="102"/>
+      <c r="R22" s="98"/>
+      <c r="S22" s="99"/>
+      <c r="T22" s="98"/>
+      <c r="U22" s="80"/>
+      <c r="V22" s="80"/>
+      <c r="W22" s="99"/>
+      <c r="X22" s="98"/>
+      <c r="Y22" s="99"/>
     </row>
     <row r="23" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B23" s="45"/>
-      <c r="C23" s="109"/>
-      <c r="D23" s="111"/>
-      <c r="E23" s="111"/>
-      <c r="F23" s="110"/>
-      <c r="G23" s="109"/>
-      <c r="H23" s="111"/>
-      <c r="I23" s="111"/>
-      <c r="J23" s="110"/>
-      <c r="K23" s="112"/>
-      <c r="L23" s="107"/>
-      <c r="M23" s="107"/>
-      <c r="N23" s="107"/>
-      <c r="O23" s="107"/>
-      <c r="P23" s="107"/>
-      <c r="Q23" s="108"/>
-      <c r="R23" s="109"/>
-      <c r="S23" s="110"/>
-      <c r="T23" s="109"/>
-      <c r="U23" s="111"/>
-      <c r="V23" s="111"/>
-      <c r="W23" s="110"/>
-      <c r="X23" s="109"/>
-      <c r="Y23" s="110"/>
+      <c r="C23" s="98"/>
+      <c r="D23" s="80"/>
+      <c r="E23" s="80"/>
+      <c r="F23" s="99"/>
+      <c r="G23" s="98"/>
+      <c r="H23" s="80"/>
+      <c r="I23" s="80"/>
+      <c r="J23" s="99"/>
+      <c r="K23" s="100"/>
+      <c r="L23" s="101"/>
+      <c r="M23" s="101"/>
+      <c r="N23" s="101"/>
+      <c r="O23" s="101"/>
+      <c r="P23" s="101"/>
+      <c r="Q23" s="102"/>
+      <c r="R23" s="98"/>
+      <c r="S23" s="99"/>
+      <c r="T23" s="98"/>
+      <c r="U23" s="80"/>
+      <c r="V23" s="80"/>
+      <c r="W23" s="99"/>
+      <c r="X23" s="98"/>
+      <c r="Y23" s="99"/>
     </row>
     <row r="24" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B24" s="45"/>
-      <c r="C24" s="109"/>
-      <c r="D24" s="111"/>
-      <c r="E24" s="111"/>
-      <c r="F24" s="110"/>
-      <c r="G24" s="109"/>
-      <c r="H24" s="111"/>
-      <c r="I24" s="111"/>
-      <c r="J24" s="110"/>
-      <c r="K24" s="112"/>
-      <c r="L24" s="107"/>
-      <c r="M24" s="107"/>
-      <c r="N24" s="107"/>
-      <c r="O24" s="107"/>
-      <c r="P24" s="107"/>
-      <c r="Q24" s="108"/>
-      <c r="R24" s="109"/>
-      <c r="S24" s="110"/>
-      <c r="T24" s="109"/>
-      <c r="U24" s="111"/>
-      <c r="V24" s="111"/>
-      <c r="W24" s="110"/>
-      <c r="X24" s="109"/>
-      <c r="Y24" s="110"/>
+      <c r="C24" s="98"/>
+      <c r="D24" s="80"/>
+      <c r="E24" s="80"/>
+      <c r="F24" s="99"/>
+      <c r="G24" s="98"/>
+      <c r="H24" s="80"/>
+      <c r="I24" s="80"/>
+      <c r="J24" s="99"/>
+      <c r="K24" s="100"/>
+      <c r="L24" s="101"/>
+      <c r="M24" s="101"/>
+      <c r="N24" s="101"/>
+      <c r="O24" s="101"/>
+      <c r="P24" s="101"/>
+      <c r="Q24" s="102"/>
+      <c r="R24" s="98"/>
+      <c r="S24" s="99"/>
+      <c r="T24" s="98"/>
+      <c r="U24" s="80"/>
+      <c r="V24" s="80"/>
+      <c r="W24" s="99"/>
+      <c r="X24" s="98"/>
+      <c r="Y24" s="99"/>
     </row>
     <row r="25" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B25" s="45"/>
-      <c r="C25" s="109"/>
-      <c r="D25" s="111"/>
-      <c r="E25" s="111"/>
-      <c r="F25" s="110"/>
-      <c r="G25" s="109"/>
-      <c r="H25" s="111"/>
-      <c r="I25" s="111"/>
-      <c r="J25" s="110"/>
-      <c r="K25" s="112"/>
-      <c r="L25" s="107"/>
-      <c r="M25" s="107"/>
-      <c r="N25" s="107"/>
-      <c r="O25" s="107"/>
-      <c r="P25" s="107"/>
-      <c r="Q25" s="108"/>
-      <c r="R25" s="109"/>
-      <c r="S25" s="110"/>
-      <c r="T25" s="109"/>
-      <c r="U25" s="111"/>
-      <c r="V25" s="111"/>
-      <c r="W25" s="110"/>
-      <c r="X25" s="109"/>
-      <c r="Y25" s="110"/>
+      <c r="C25" s="98"/>
+      <c r="D25" s="80"/>
+      <c r="E25" s="80"/>
+      <c r="F25" s="99"/>
+      <c r="G25" s="98"/>
+      <c r="H25" s="80"/>
+      <c r="I25" s="80"/>
+      <c r="J25" s="99"/>
+      <c r="K25" s="100"/>
+      <c r="L25" s="101"/>
+      <c r="M25" s="101"/>
+      <c r="N25" s="101"/>
+      <c r="O25" s="101"/>
+      <c r="P25" s="101"/>
+      <c r="Q25" s="102"/>
+      <c r="R25" s="98"/>
+      <c r="S25" s="99"/>
+      <c r="T25" s="98"/>
+      <c r="U25" s="80"/>
+      <c r="V25" s="80"/>
+      <c r="W25" s="99"/>
+      <c r="X25" s="98"/>
+      <c r="Y25" s="99"/>
     </row>
     <row r="26" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B26" s="45"/>
-      <c r="C26" s="109"/>
-      <c r="D26" s="111"/>
-      <c r="E26" s="111"/>
-      <c r="F26" s="110"/>
-      <c r="G26" s="109"/>
-      <c r="H26" s="111"/>
-      <c r="I26" s="111"/>
-      <c r="J26" s="110"/>
-      <c r="K26" s="112"/>
-      <c r="L26" s="107"/>
-      <c r="M26" s="107"/>
-      <c r="N26" s="107"/>
-      <c r="O26" s="107"/>
-      <c r="P26" s="107"/>
-      <c r="Q26" s="108"/>
-      <c r="R26" s="109"/>
-      <c r="S26" s="110"/>
-      <c r="T26" s="109"/>
-      <c r="U26" s="111"/>
-      <c r="V26" s="111"/>
-      <c r="W26" s="110"/>
-      <c r="X26" s="109"/>
-      <c r="Y26" s="110"/>
+      <c r="C26" s="98"/>
+      <c r="D26" s="80"/>
+      <c r="E26" s="80"/>
+      <c r="F26" s="99"/>
+      <c r="G26" s="98"/>
+      <c r="H26" s="80"/>
+      <c r="I26" s="80"/>
+      <c r="J26" s="99"/>
+      <c r="K26" s="100"/>
+      <c r="L26" s="101"/>
+      <c r="M26" s="101"/>
+      <c r="N26" s="101"/>
+      <c r="O26" s="101"/>
+      <c r="P26" s="101"/>
+      <c r="Q26" s="102"/>
+      <c r="R26" s="98"/>
+      <c r="S26" s="99"/>
+      <c r="T26" s="98"/>
+      <c r="U26" s="80"/>
+      <c r="V26" s="80"/>
+      <c r="W26" s="99"/>
+      <c r="X26" s="98"/>
+      <c r="Y26" s="99"/>
     </row>
     <row r="27" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B27" s="45"/>
-      <c r="C27" s="109"/>
-      <c r="D27" s="111"/>
-      <c r="E27" s="111"/>
-      <c r="F27" s="110"/>
-      <c r="G27" s="109"/>
-      <c r="H27" s="111"/>
-      <c r="I27" s="111"/>
-      <c r="J27" s="110"/>
-      <c r="K27" s="112"/>
-      <c r="L27" s="107"/>
-      <c r="M27" s="107"/>
-      <c r="N27" s="107"/>
-      <c r="O27" s="107"/>
-      <c r="P27" s="107"/>
-      <c r="Q27" s="108"/>
-      <c r="R27" s="109"/>
-      <c r="S27" s="110"/>
-      <c r="T27" s="109"/>
-      <c r="U27" s="111"/>
-      <c r="V27" s="111"/>
-      <c r="W27" s="110"/>
-      <c r="X27" s="109"/>
-      <c r="Y27" s="110"/>
+      <c r="C27" s="98"/>
+      <c r="D27" s="80"/>
+      <c r="E27" s="80"/>
+      <c r="F27" s="99"/>
+      <c r="G27" s="98"/>
+      <c r="H27" s="80"/>
+      <c r="I27" s="80"/>
+      <c r="J27" s="99"/>
+      <c r="K27" s="100"/>
+      <c r="L27" s="101"/>
+      <c r="M27" s="101"/>
+      <c r="N27" s="101"/>
+      <c r="O27" s="101"/>
+      <c r="P27" s="101"/>
+      <c r="Q27" s="102"/>
+      <c r="R27" s="98"/>
+      <c r="S27" s="99"/>
+      <c r="T27" s="98"/>
+      <c r="U27" s="80"/>
+      <c r="V27" s="80"/>
+      <c r="W27" s="99"/>
+      <c r="X27" s="98"/>
+      <c r="Y27" s="99"/>
     </row>
     <row r="28" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B28" s="45"/>
-      <c r="C28" s="109"/>
-      <c r="D28" s="111"/>
-      <c r="E28" s="111"/>
-      <c r="F28" s="110"/>
-      <c r="G28" s="109"/>
-      <c r="H28" s="111"/>
-      <c r="I28" s="111"/>
-      <c r="J28" s="110"/>
-      <c r="K28" s="112"/>
-      <c r="L28" s="107"/>
-      <c r="M28" s="107"/>
-      <c r="N28" s="107"/>
-      <c r="O28" s="107"/>
-      <c r="P28" s="107"/>
-      <c r="Q28" s="108"/>
-      <c r="R28" s="109"/>
-      <c r="S28" s="110"/>
-      <c r="T28" s="109"/>
-      <c r="U28" s="111"/>
-      <c r="V28" s="111"/>
-      <c r="W28" s="110"/>
-      <c r="X28" s="109"/>
-      <c r="Y28" s="110"/>
+      <c r="C28" s="98"/>
+      <c r="D28" s="80"/>
+      <c r="E28" s="80"/>
+      <c r="F28" s="99"/>
+      <c r="G28" s="98"/>
+      <c r="H28" s="80"/>
+      <c r="I28" s="80"/>
+      <c r="J28" s="99"/>
+      <c r="K28" s="100"/>
+      <c r="L28" s="101"/>
+      <c r="M28" s="101"/>
+      <c r="N28" s="101"/>
+      <c r="O28" s="101"/>
+      <c r="P28" s="101"/>
+      <c r="Q28" s="102"/>
+      <c r="R28" s="98"/>
+      <c r="S28" s="99"/>
+      <c r="T28" s="98"/>
+      <c r="U28" s="80"/>
+      <c r="V28" s="80"/>
+      <c r="W28" s="99"/>
+      <c r="X28" s="98"/>
+      <c r="Y28" s="99"/>
     </row>
     <row r="29" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B29" s="45"/>
-      <c r="C29" s="109"/>
-      <c r="D29" s="111"/>
-      <c r="E29" s="111"/>
-      <c r="F29" s="110"/>
-      <c r="G29" s="109"/>
-      <c r="H29" s="111"/>
-      <c r="I29" s="111"/>
-      <c r="J29" s="110"/>
-      <c r="K29" s="112"/>
-      <c r="L29" s="107"/>
-      <c r="M29" s="107"/>
-      <c r="N29" s="107"/>
-      <c r="O29" s="107"/>
-      <c r="P29" s="107"/>
-      <c r="Q29" s="108"/>
-      <c r="R29" s="109"/>
-      <c r="S29" s="110"/>
-      <c r="T29" s="109"/>
-      <c r="U29" s="111"/>
-      <c r="V29" s="111"/>
-      <c r="W29" s="110"/>
-      <c r="X29" s="109"/>
-      <c r="Y29" s="110"/>
+      <c r="C29" s="98"/>
+      <c r="D29" s="80"/>
+      <c r="E29" s="80"/>
+      <c r="F29" s="99"/>
+      <c r="G29" s="98"/>
+      <c r="H29" s="80"/>
+      <c r="I29" s="80"/>
+      <c r="J29" s="99"/>
+      <c r="K29" s="100"/>
+      <c r="L29" s="101"/>
+      <c r="M29" s="101"/>
+      <c r="N29" s="101"/>
+      <c r="O29" s="101"/>
+      <c r="P29" s="101"/>
+      <c r="Q29" s="102"/>
+      <c r="R29" s="98"/>
+      <c r="S29" s="99"/>
+      <c r="T29" s="98"/>
+      <c r="U29" s="80"/>
+      <c r="V29" s="80"/>
+      <c r="W29" s="99"/>
+      <c r="X29" s="98"/>
+      <c r="Y29" s="99"/>
     </row>
     <row r="30" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="44" t="s">
         <v>311</v>
       </c>
       <c r="B30" s="45"/>
-      <c r="C30" s="109"/>
-      <c r="D30" s="111"/>
-      <c r="E30" s="111"/>
-      <c r="F30" s="110"/>
-      <c r="G30" s="109"/>
-      <c r="H30" s="111"/>
-      <c r="I30" s="111"/>
-      <c r="J30" s="110"/>
-      <c r="K30" s="112"/>
-      <c r="L30" s="107"/>
-      <c r="M30" s="107"/>
-      <c r="N30" s="107"/>
-      <c r="O30" s="107"/>
-      <c r="P30" s="107"/>
-      <c r="Q30" s="108"/>
-      <c r="R30" s="109"/>
-      <c r="S30" s="110"/>
-      <c r="T30" s="109"/>
-      <c r="U30" s="111"/>
-      <c r="V30" s="111"/>
-      <c r="W30" s="110"/>
-      <c r="X30" s="109"/>
-      <c r="Y30" s="110"/>
+      <c r="C30" s="98"/>
+      <c r="D30" s="80"/>
+      <c r="E30" s="80"/>
+      <c r="F30" s="99"/>
+      <c r="G30" s="98"/>
+      <c r="H30" s="80"/>
+      <c r="I30" s="80"/>
+      <c r="J30" s="99"/>
+      <c r="K30" s="100"/>
+      <c r="L30" s="101"/>
+      <c r="M30" s="101"/>
+      <c r="N30" s="101"/>
+      <c r="O30" s="101"/>
+      <c r="P30" s="101"/>
+      <c r="Q30" s="102"/>
+      <c r="R30" s="98"/>
+      <c r="S30" s="99"/>
+      <c r="T30" s="98"/>
+      <c r="U30" s="80"/>
+      <c r="V30" s="80"/>
+      <c r="W30" s="99"/>
+      <c r="X30" s="98"/>
+      <c r="Y30" s="99"/>
     </row>
     <row r="31" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="44"/>
       <c r="B31" s="45"/>
-      <c r="C31" s="97"/>
-      <c r="D31" s="98"/>
-      <c r="E31" s="98"/>
-      <c r="F31" s="99"/>
-      <c r="G31" s="97"/>
-      <c r="H31" s="98"/>
-      <c r="I31" s="98"/>
-      <c r="J31" s="99"/>
-      <c r="K31" s="112"/>
-      <c r="L31" s="107"/>
-      <c r="M31" s="107"/>
-      <c r="N31" s="107"/>
-      <c r="O31" s="107"/>
-      <c r="P31" s="107"/>
-      <c r="Q31" s="108"/>
-      <c r="R31" s="109"/>
-      <c r="S31" s="110"/>
-      <c r="T31" s="109"/>
-      <c r="U31" s="111"/>
-      <c r="V31" s="111"/>
-      <c r="W31" s="110"/>
-      <c r="X31" s="109"/>
-      <c r="Y31" s="110"/>
+      <c r="C31" s="103"/>
+      <c r="D31" s="104"/>
+      <c r="E31" s="104"/>
+      <c r="F31" s="105"/>
+      <c r="G31" s="103"/>
+      <c r="H31" s="104"/>
+      <c r="I31" s="104"/>
+      <c r="J31" s="105"/>
+      <c r="K31" s="100"/>
+      <c r="L31" s="101"/>
+      <c r="M31" s="101"/>
+      <c r="N31" s="101"/>
+      <c r="O31" s="101"/>
+      <c r="P31" s="101"/>
+      <c r="Q31" s="102"/>
+      <c r="R31" s="98"/>
+      <c r="S31" s="99"/>
+      <c r="T31" s="98"/>
+      <c r="U31" s="80"/>
+      <c r="V31" s="80"/>
+      <c r="W31" s="99"/>
+      <c r="X31" s="98"/>
+      <c r="Y31" s="99"/>
     </row>
     <row r="32" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="44"/>
       <c r="B32" s="45"/>
-      <c r="C32" s="97"/>
-      <c r="D32" s="98"/>
-      <c r="E32" s="98"/>
-      <c r="F32" s="99"/>
-      <c r="G32" s="97"/>
-      <c r="H32" s="98"/>
-      <c r="I32" s="98"/>
-      <c r="J32" s="99"/>
+      <c r="C32" s="103"/>
+      <c r="D32" s="104"/>
+      <c r="E32" s="104"/>
+      <c r="F32" s="105"/>
+      <c r="G32" s="103"/>
+      <c r="H32" s="104"/>
+      <c r="I32" s="104"/>
+      <c r="J32" s="105"/>
       <c r="K32" s="106"/>
-      <c r="L32" s="107"/>
-      <c r="M32" s="107"/>
-      <c r="N32" s="107"/>
-      <c r="O32" s="107"/>
-      <c r="P32" s="107"/>
-      <c r="Q32" s="108"/>
-      <c r="R32" s="109"/>
-      <c r="S32" s="110"/>
-      <c r="T32" s="109"/>
-      <c r="U32" s="111"/>
-      <c r="V32" s="111"/>
-      <c r="W32" s="110"/>
-      <c r="X32" s="109"/>
-      <c r="Y32" s="110"/>
+      <c r="L32" s="101"/>
+      <c r="M32" s="101"/>
+      <c r="N32" s="101"/>
+      <c r="O32" s="101"/>
+      <c r="P32" s="101"/>
+      <c r="Q32" s="102"/>
+      <c r="R32" s="98"/>
+      <c r="S32" s="99"/>
+      <c r="T32" s="98"/>
+      <c r="U32" s="80"/>
+      <c r="V32" s="80"/>
+      <c r="W32" s="99"/>
+      <c r="X32" s="98"/>
+      <c r="Y32" s="99"/>
     </row>
     <row r="33" spans="1:25" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="46"/>
       <c r="B33" s="47"/>
-      <c r="C33" s="97"/>
-      <c r="D33" s="98"/>
-      <c r="E33" s="98"/>
-      <c r="F33" s="99"/>
-      <c r="G33" s="97"/>
-      <c r="H33" s="98"/>
-      <c r="I33" s="98"/>
-      <c r="J33" s="99"/>
-      <c r="K33" s="100"/>
-      <c r="L33" s="101"/>
-      <c r="M33" s="101"/>
-      <c r="N33" s="101"/>
-      <c r="O33" s="101"/>
-      <c r="P33" s="101"/>
-      <c r="Q33" s="102"/>
-      <c r="R33" s="103"/>
-      <c r="S33" s="104"/>
-      <c r="T33" s="103"/>
-      <c r="U33" s="105"/>
-      <c r="V33" s="105"/>
-      <c r="W33" s="104"/>
-      <c r="X33" s="103"/>
-      <c r="Y33" s="104"/>
+      <c r="C33" s="103"/>
+      <c r="D33" s="104"/>
+      <c r="E33" s="104"/>
+      <c r="F33" s="105"/>
+      <c r="G33" s="103"/>
+      <c r="H33" s="104"/>
+      <c r="I33" s="104"/>
+      <c r="J33" s="105"/>
+      <c r="K33" s="124"/>
+      <c r="L33" s="125"/>
+      <c r="M33" s="125"/>
+      <c r="N33" s="125"/>
+      <c r="O33" s="125"/>
+      <c r="P33" s="125"/>
+      <c r="Q33" s="126"/>
+      <c r="R33" s="127"/>
+      <c r="S33" s="128"/>
+      <c r="T33" s="127"/>
+      <c r="U33" s="129"/>
+      <c r="V33" s="129"/>
+      <c r="W33" s="128"/>
+      <c r="X33" s="127"/>
+      <c r="Y33" s="128"/>
     </row>
     <row r="34" spans="1:25" ht="41.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="80" t="s">
+      <c r="A34" s="107" t="s">
         <v>312</v>
       </c>
-      <c r="B34" s="81"/>
-      <c r="C34" s="84" t="s">
+      <c r="B34" s="108"/>
+      <c r="C34" s="111" t="s">
         <v>313</v>
       </c>
-      <c r="D34" s="85"/>
-      <c r="E34" s="85"/>
-      <c r="F34" s="86"/>
-      <c r="G34" s="84" t="s">
+      <c r="D34" s="112"/>
+      <c r="E34" s="112"/>
+      <c r="F34" s="113"/>
+      <c r="G34" s="111" t="s">
         <v>314</v>
       </c>
-      <c r="H34" s="85"/>
-      <c r="I34" s="85"/>
-      <c r="J34" s="86"/>
-      <c r="K34" s="80" t="s">
+      <c r="H34" s="112"/>
+      <c r="I34" s="112"/>
+      <c r="J34" s="113"/>
+      <c r="K34" s="107" t="s">
         <v>315</v>
       </c>
-      <c r="L34" s="90"/>
-      <c r="M34" s="90"/>
-      <c r="N34" s="90"/>
-      <c r="O34" s="90"/>
-      <c r="P34" s="90"/>
-      <c r="Q34" s="91"/>
-      <c r="R34" s="80" t="s">
+      <c r="L34" s="117"/>
+      <c r="M34" s="117"/>
+      <c r="N34" s="117"/>
+      <c r="O34" s="117"/>
+      <c r="P34" s="117"/>
+      <c r="Q34" s="118"/>
+      <c r="R34" s="107" t="s">
         <v>316</v>
       </c>
-      <c r="S34" s="81"/>
-      <c r="T34" s="80" t="s">
+      <c r="S34" s="108"/>
+      <c r="T34" s="107" t="s">
         <v>317</v>
       </c>
-      <c r="U34" s="95"/>
-      <c r="V34" s="95"/>
-      <c r="W34" s="81"/>
-      <c r="X34" s="80" t="s">
+      <c r="U34" s="122"/>
+      <c r="V34" s="122"/>
+      <c r="W34" s="108"/>
+      <c r="X34" s="107" t="s">
         <v>318</v>
       </c>
-      <c r="Y34" s="81"/>
+      <c r="Y34" s="108"/>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A35" s="82"/>
-      <c r="B35" s="83"/>
-      <c r="C35" s="87"/>
-      <c r="D35" s="88"/>
-      <c r="E35" s="88"/>
-      <c r="F35" s="89"/>
-      <c r="G35" s="87"/>
-      <c r="H35" s="88"/>
-      <c r="I35" s="88"/>
-      <c r="J35" s="89"/>
-      <c r="K35" s="92"/>
-      <c r="L35" s="93"/>
-      <c r="M35" s="93"/>
-      <c r="N35" s="93"/>
-      <c r="O35" s="93"/>
-      <c r="P35" s="93"/>
-      <c r="Q35" s="94"/>
-      <c r="R35" s="82"/>
-      <c r="S35" s="83"/>
-      <c r="T35" s="82"/>
-      <c r="U35" s="96"/>
-      <c r="V35" s="96"/>
-      <c r="W35" s="83"/>
-      <c r="X35" s="82"/>
-      <c r="Y35" s="83"/>
+      <c r="A35" s="109"/>
+      <c r="B35" s="110"/>
+      <c r="C35" s="114"/>
+      <c r="D35" s="115"/>
+      <c r="E35" s="115"/>
+      <c r="F35" s="116"/>
+      <c r="G35" s="114"/>
+      <c r="H35" s="115"/>
+      <c r="I35" s="115"/>
+      <c r="J35" s="116"/>
+      <c r="K35" s="119"/>
+      <c r="L35" s="120"/>
+      <c r="M35" s="120"/>
+      <c r="N35" s="120"/>
+      <c r="O35" s="120"/>
+      <c r="P35" s="120"/>
+      <c r="Q35" s="121"/>
+      <c r="R35" s="109"/>
+      <c r="S35" s="110"/>
+      <c r="T35" s="109"/>
+      <c r="U35" s="123"/>
+      <c r="V35" s="123"/>
+      <c r="W35" s="110"/>
+      <c r="X35" s="109"/>
+      <c r="Y35" s="110"/>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A36" s="48" t="s">
@@ -11401,15 +11402,116 @@
     </row>
   </sheetData>
   <mergeCells count="143">
-    <mergeCell ref="P12:R12"/>
-    <mergeCell ref="O7:Q8"/>
-    <mergeCell ref="R7:T8"/>
-    <mergeCell ref="U7:W8"/>
-    <mergeCell ref="P10:R10"/>
-    <mergeCell ref="S10:W10"/>
-    <mergeCell ref="P11:R11"/>
-    <mergeCell ref="S11:W11"/>
-    <mergeCell ref="P1:V1"/>
+    <mergeCell ref="X34:Y35"/>
+    <mergeCell ref="A34:B35"/>
+    <mergeCell ref="C34:F35"/>
+    <mergeCell ref="G34:J35"/>
+    <mergeCell ref="K34:Q35"/>
+    <mergeCell ref="R34:S35"/>
+    <mergeCell ref="T34:W35"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="G33:J33"/>
+    <mergeCell ref="K33:Q33"/>
+    <mergeCell ref="R33:S33"/>
+    <mergeCell ref="T33:W33"/>
+    <mergeCell ref="X33:Y33"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="G32:J32"/>
+    <mergeCell ref="K32:Q32"/>
+    <mergeCell ref="R32:S32"/>
+    <mergeCell ref="T32:W32"/>
+    <mergeCell ref="X32:Y32"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="G31:J31"/>
+    <mergeCell ref="K31:Q31"/>
+    <mergeCell ref="R31:S31"/>
+    <mergeCell ref="T31:W31"/>
+    <mergeCell ref="X31:Y31"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="G30:J30"/>
+    <mergeCell ref="K30:Q30"/>
+    <mergeCell ref="R30:S30"/>
+    <mergeCell ref="T30:W30"/>
+    <mergeCell ref="X30:Y30"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="G29:J29"/>
+    <mergeCell ref="K29:Q29"/>
+    <mergeCell ref="R29:S29"/>
+    <mergeCell ref="T29:W29"/>
+    <mergeCell ref="X29:Y29"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="G28:J28"/>
+    <mergeCell ref="K28:Q28"/>
+    <mergeCell ref="R28:S28"/>
+    <mergeCell ref="T28:W28"/>
+    <mergeCell ref="X28:Y28"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="G27:J27"/>
+    <mergeCell ref="K27:Q27"/>
+    <mergeCell ref="R27:S27"/>
+    <mergeCell ref="T27:W27"/>
+    <mergeCell ref="X27:Y27"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="G26:J26"/>
+    <mergeCell ref="K26:Q26"/>
+    <mergeCell ref="R26:S26"/>
+    <mergeCell ref="T26:W26"/>
+    <mergeCell ref="X26:Y26"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="G25:J25"/>
+    <mergeCell ref="K25:Q25"/>
+    <mergeCell ref="R25:S25"/>
+    <mergeCell ref="T25:W25"/>
+    <mergeCell ref="X25:Y25"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="G24:J24"/>
+    <mergeCell ref="K24:Q24"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="T24:W24"/>
+    <mergeCell ref="X24:Y24"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="G23:J23"/>
+    <mergeCell ref="K23:Q23"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="T23:W23"/>
+    <mergeCell ref="X23:Y23"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="G22:J22"/>
+    <mergeCell ref="K22:Q22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="T22:W22"/>
+    <mergeCell ref="X22:Y22"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="G21:J21"/>
+    <mergeCell ref="K21:Q21"/>
+    <mergeCell ref="R21:S21"/>
+    <mergeCell ref="T21:W21"/>
+    <mergeCell ref="X21:Y21"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="G20:J20"/>
+    <mergeCell ref="K20:Q20"/>
+    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="T20:W20"/>
+    <mergeCell ref="X20:Y20"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="G19:J19"/>
+    <mergeCell ref="K19:Q19"/>
+    <mergeCell ref="R19:S19"/>
+    <mergeCell ref="T19:W19"/>
+    <mergeCell ref="X19:Y19"/>
+    <mergeCell ref="T14:W14"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="G18:J18"/>
+    <mergeCell ref="K18:Q18"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="T18:W18"/>
+    <mergeCell ref="X18:Y18"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="G17:J17"/>
+    <mergeCell ref="K17:Q17"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="T17:W17"/>
+    <mergeCell ref="X17:Y17"/>
     <mergeCell ref="X1:Y1"/>
     <mergeCell ref="D2:W2"/>
     <mergeCell ref="D3:W3"/>
@@ -11434,116 +11536,15 @@
     <mergeCell ref="G14:J14"/>
     <mergeCell ref="K14:Q14"/>
     <mergeCell ref="R14:S14"/>
-    <mergeCell ref="T14:W14"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="G18:J18"/>
-    <mergeCell ref="K18:Q18"/>
-    <mergeCell ref="R18:S18"/>
-    <mergeCell ref="T18:W18"/>
-    <mergeCell ref="X18:Y18"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="G17:J17"/>
-    <mergeCell ref="K17:Q17"/>
-    <mergeCell ref="R17:S17"/>
-    <mergeCell ref="T17:W17"/>
-    <mergeCell ref="X17:Y17"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="G20:J20"/>
-    <mergeCell ref="K20:Q20"/>
-    <mergeCell ref="R20:S20"/>
-    <mergeCell ref="T20:W20"/>
-    <mergeCell ref="X20:Y20"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="G19:J19"/>
-    <mergeCell ref="K19:Q19"/>
-    <mergeCell ref="R19:S19"/>
-    <mergeCell ref="T19:W19"/>
-    <mergeCell ref="X19:Y19"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="G22:J22"/>
-    <mergeCell ref="K22:Q22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="T22:W22"/>
-    <mergeCell ref="X22:Y22"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="G21:J21"/>
-    <mergeCell ref="K21:Q21"/>
-    <mergeCell ref="R21:S21"/>
-    <mergeCell ref="T21:W21"/>
-    <mergeCell ref="X21:Y21"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="G24:J24"/>
-    <mergeCell ref="K24:Q24"/>
-    <mergeCell ref="R24:S24"/>
-    <mergeCell ref="T24:W24"/>
-    <mergeCell ref="X24:Y24"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="G23:J23"/>
-    <mergeCell ref="K23:Q23"/>
-    <mergeCell ref="R23:S23"/>
-    <mergeCell ref="T23:W23"/>
-    <mergeCell ref="X23:Y23"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="G26:J26"/>
-    <mergeCell ref="K26:Q26"/>
-    <mergeCell ref="R26:S26"/>
-    <mergeCell ref="T26:W26"/>
-    <mergeCell ref="X26:Y26"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="G25:J25"/>
-    <mergeCell ref="K25:Q25"/>
-    <mergeCell ref="R25:S25"/>
-    <mergeCell ref="T25:W25"/>
-    <mergeCell ref="X25:Y25"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="G28:J28"/>
-    <mergeCell ref="K28:Q28"/>
-    <mergeCell ref="R28:S28"/>
-    <mergeCell ref="T28:W28"/>
-    <mergeCell ref="X28:Y28"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="G27:J27"/>
-    <mergeCell ref="K27:Q27"/>
-    <mergeCell ref="R27:S27"/>
-    <mergeCell ref="T27:W27"/>
-    <mergeCell ref="X27:Y27"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="G30:J30"/>
-    <mergeCell ref="K30:Q30"/>
-    <mergeCell ref="R30:S30"/>
-    <mergeCell ref="T30:W30"/>
-    <mergeCell ref="X30:Y30"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="G29:J29"/>
-    <mergeCell ref="K29:Q29"/>
-    <mergeCell ref="R29:S29"/>
-    <mergeCell ref="T29:W29"/>
-    <mergeCell ref="X29:Y29"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="G32:J32"/>
-    <mergeCell ref="K32:Q32"/>
-    <mergeCell ref="R32:S32"/>
-    <mergeCell ref="T32:W32"/>
-    <mergeCell ref="X32:Y32"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="G31:J31"/>
-    <mergeCell ref="K31:Q31"/>
-    <mergeCell ref="R31:S31"/>
-    <mergeCell ref="T31:W31"/>
-    <mergeCell ref="X31:Y31"/>
-    <mergeCell ref="X34:Y35"/>
-    <mergeCell ref="A34:B35"/>
-    <mergeCell ref="C34:F35"/>
-    <mergeCell ref="G34:J35"/>
-    <mergeCell ref="K34:Q35"/>
-    <mergeCell ref="R34:S35"/>
-    <mergeCell ref="T34:W35"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="G33:J33"/>
-    <mergeCell ref="K33:Q33"/>
-    <mergeCell ref="R33:S33"/>
-    <mergeCell ref="T33:W33"/>
-    <mergeCell ref="X33:Y33"/>
+    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="O7:Q8"/>
+    <mergeCell ref="R7:T8"/>
+    <mergeCell ref="U7:W8"/>
+    <mergeCell ref="P10:R10"/>
+    <mergeCell ref="S10:W10"/>
+    <mergeCell ref="P11:R11"/>
+    <mergeCell ref="S11:W11"/>
+    <mergeCell ref="P1:V1"/>
   </mergeCells>
   <phoneticPr fontId="1"/>
   <pageMargins left="0.86614173228346458" right="0.51181102362204722" top="0.59055118110236227" bottom="0.19685039370078741" header="0.59055118110236227" footer="0.19685039370078741"/>

</xml_diff>

<commit_message>
sync(workvault): 2026-10-23 18:14 差分 5 件
</commit_message>
<xml_diff>
--- a/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/Pana-CIM管理手順書案_未承認.xlsx
+++ b/workvault-sync/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/Pana-CIM管理手順書案_未承認.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nk365-my.sharepoint.com/personal/ss80751_ad_nkc_co_jp/Documents/ドキュメント/Work_Vault/10_業務全般/PanaCIM_LNB/01_成果物/20261015_管理手順書案/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10562" documentId="13_ncr:1_{22133521-4050-492C-8145-0AE2EA6E1C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7262B560-2756-4609-88E1-6181B043A5FC}"/>
+  <xr:revisionPtr revIDLastSave="10571" documentId="13_ncr:1_{22133521-4050-492C-8145-0AE2EA6E1C2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6822FB3-74A6-4247-A275-5810271DAE47}"/>
   <bookViews>
     <workbookView xWindow="1116" yWindow="1116" windowWidth="17280" windowHeight="10500" firstSheet="12" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -7411,14 +7411,14 @@
     <xdr:from>
       <xdr:col>12</xdr:col>
       <xdr:colOff>97155</xdr:colOff>
-      <xdr:row>97</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>10160</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>41453</xdr:colOff>
-      <xdr:row>97</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>10160</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -7433,7 +7433,7 @@
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1651635" y="16268700"/>
+          <a:off x="1651635" y="15913100"/>
           <a:ext cx="462458" cy="0"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
@@ -7472,8 +7472,8 @@
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>41453</xdr:colOff>
-      <xdr:row>97</xdr:row>
-      <xdr:rowOff>45720</xdr:rowOff>
+      <xdr:row>95</xdr:row>
+      <xdr:rowOff>10160</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
@@ -7489,7 +7489,7 @@
       <xdr:spPr>
         <a:xfrm flipV="1">
           <a:off x="2114093" y="12420600"/>
-          <a:ext cx="0" cy="3848100"/>
+          <a:ext cx="0" cy="3492500"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -7498,62 +7498,6 @@
           <a:solidFill>
             <a:srgbClr val="000000"/>
           </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>41453</xdr:colOff>
-      <xdr:row>73</xdr:row>
-      <xdr:rowOff>60960</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>17</xdr:col>
-      <xdr:colOff>44044</xdr:colOff>
-      <xdr:row>73</xdr:row>
-      <xdr:rowOff>60960</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="58" name="直線矢印コネクタ 57">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6FFDCE70-2121-69C6-F2E7-C5AE17056E00}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipH="1">
-          <a:off x="2114093" y="12420600"/>
-          <a:ext cx="132131" cy="0"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="000000"/>
-          </a:solidFill>
-          <a:tailEnd type="triangle"/>
         </a:ln>
       </xdr:spPr>
       <xdr:style>
@@ -9480,6 +9424,62 @@
     </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>41453</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>44044</xdr:colOff>
+      <xdr:row>73</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="5" name="Straight Arrow Connector 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EBA0C8A6-D7E4-3171-86D9-D5D83986E374}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2114093" y="12420600"/>
+          <a:ext cx="132131" cy="0"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>